<commit_message>
Redesign summary as month-only dashboard with Apr 2026-Apr 2029 timeline
Co-authored-by: Samuel Kafui Kwawukume <samkafs@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/personal_finance_tracker.xlsx
+++ b/personal_finance_tracker.xlsx
@@ -23,10 +23,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="165" formatCode="$#,##0.00"/>
     <numFmt numFmtId="166" formatCode="&quot;GHS&quot; #,##0.00"/>
+    <numFmt numFmtId="167" formatCode="mmm yyyy"/>
   </numFmts>
   <fonts count="6">
     <font>
@@ -95,7 +96,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -117,6 +118,7 @@
     <xf numFmtId="165" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -482,44 +484,43 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H29"/>
+  <dimension ref="A1:M66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="40" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="20" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Monthly Finance Dashboard</t>
+          <t>Monthly Flow Dashboard (Month-Only)</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Month</t>
+          <t>Selected Month (enter any date):</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="C3" s="14" t="n">
+        <v>46113</v>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Enter any date in month</t>
-        </is>
-      </c>
-      <c r="C3" s="14" t="inlineStr">
-        <is>
-          <t>2026-04-01</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>How to use every month</t>
+          <t>How it works</t>
         </is>
       </c>
     </row>
@@ -542,28 +543,28 @@
         <f>EOMONTH(C3,0)</f>
         <v/>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
-          <t>1) In C3, enter any date in target month</t>
+          <t>1) Change C3 to any date in a month</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="H5" t="inlineStr">
+      <c r="J5" t="inlineStr">
         <is>
-          <t>2) Keep adding dated transactions in tabs</t>
+          <t>2) Selected-month tables update automatically</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>USD Bank Accounts</t>
+          <t>Selected Month - USD Bank Accounts</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="J6" t="inlineStr">
         <is>
-          <t>3) Monthly totals auto-filter by C3 month</t>
+          <t>3) Timeline is auto-filled Apr 2026-Apr 2029</t>
         </is>
       </c>
     </row>
@@ -575,32 +576,27 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Current Balance (USD)</t>
+          <t>Money In</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>Month In</t>
+          <t>Money Out</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>Month Out</t>
+          <t>Tax</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>Month Tax</t>
+          <t>Net Flow</t>
         </is>
       </c>
-      <c r="F7" s="5" t="inlineStr">
+      <c r="J7" t="inlineStr">
         <is>
-          <t>Net Month Change</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>4) No new file needed each month</t>
+          <t>4) No current balance columns are shown</t>
         </is>
       </c>
     </row>
@@ -611,29 +607,20 @@
         </is>
       </c>
       <c r="B8" s="15">
-        <f>'Current'!B4</f>
+        <f>SUMIFS('Current'!D:D,'Current'!A:A,"&gt;="&amp;$B$4,'Current'!A:A,"&lt;="&amp;$D$4)</f>
         <v/>
       </c>
       <c r="C8" s="15">
-        <f>SUMIFS('Current'!D:D,'Current'!A:A,"&gt;="&amp;$B$4,'Current'!A:A,"&lt;="&amp;$D$4)</f>
+        <f>SUMIFS('Current'!E:E,'Current'!A:A,"&gt;="&amp;$B$4,'Current'!A:A,"&lt;="&amp;$D$4)</f>
         <v/>
       </c>
       <c r="D8" s="15">
-        <f>SUMIFS('Current'!E:E,'Current'!A:A,"&gt;="&amp;$B$4,'Current'!A:A,"&lt;="&amp;$D$4)</f>
+        <f>SUMIFS('Current'!F:F,'Current'!A:A,"&gt;="&amp;$B$4,'Current'!A:A,"&lt;="&amp;$D$4)</f>
         <v/>
       </c>
       <c r="E8" s="15">
-        <f>SUMIFS('Current'!F:F,'Current'!A:A,"&gt;="&amp;$B$4,'Current'!A:A,"&lt;="&amp;$D$4)</f>
-        <v/>
-      </c>
-      <c r="F8" s="15">
-        <f>C8-D8-E8</f>
-        <v/>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>5) Credit cards: Payment reduces owed</t>
-        </is>
+        <f>B8-C8-D8</f>
+        <v/>
       </c>
     </row>
     <row r="9">
@@ -643,29 +630,20 @@
         </is>
       </c>
       <c r="B9" s="15">
-        <f>'Chase'!B4</f>
+        <f>SUMIFS('Chase'!D:D,'Chase'!A:A,"&gt;="&amp;$B$4,'Chase'!A:A,"&lt;="&amp;$D$4)</f>
         <v/>
       </c>
       <c r="C9" s="15">
-        <f>SUMIFS('Chase'!D:D,'Chase'!A:A,"&gt;="&amp;$B$4,'Chase'!A:A,"&lt;="&amp;$D$4)</f>
+        <f>SUMIFS('Chase'!E:E,'Chase'!A:A,"&gt;="&amp;$B$4,'Chase'!A:A,"&lt;="&amp;$D$4)</f>
         <v/>
       </c>
       <c r="D9" s="15">
-        <f>SUMIFS('Chase'!E:E,'Chase'!A:A,"&gt;="&amp;$B$4,'Chase'!A:A,"&lt;="&amp;$D$4)</f>
+        <f>SUMIFS('Chase'!F:F,'Chase'!A:A,"&gt;="&amp;$B$4,'Chase'!A:A,"&lt;="&amp;$D$4)</f>
         <v/>
       </c>
       <c r="E9" s="15">
-        <f>SUMIFS('Chase'!F:F,'Chase'!A:A,"&gt;="&amp;$B$4,'Chase'!A:A,"&lt;="&amp;$D$4)</f>
-        <v/>
-      </c>
-      <c r="F9" s="15">
-        <f>C9-D9-E9</f>
-        <v/>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>6) Credit cards: Spend/Tax increase owed</t>
-        </is>
+        <f>B9-C9-D9</f>
+        <v/>
       </c>
     </row>
     <row r="10">
@@ -675,23 +653,19 @@
         </is>
       </c>
       <c r="B10" s="15">
-        <f>'Wellsfargo'!B4</f>
+        <f>SUMIFS('Wellsfargo'!D:D,'Wellsfargo'!A:A,"&gt;="&amp;$B$4,'Wellsfargo'!A:A,"&lt;="&amp;$D$4)</f>
         <v/>
       </c>
       <c r="C10" s="15">
-        <f>SUMIFS('Wellsfargo'!D:D,'Wellsfargo'!A:A,"&gt;="&amp;$B$4,'Wellsfargo'!A:A,"&lt;="&amp;$D$4)</f>
+        <f>SUMIFS('Wellsfargo'!E:E,'Wellsfargo'!A:A,"&gt;="&amp;$B$4,'Wellsfargo'!A:A,"&lt;="&amp;$D$4)</f>
         <v/>
       </c>
       <c r="D10" s="15">
-        <f>SUMIFS('Wellsfargo'!E:E,'Wellsfargo'!A:A,"&gt;="&amp;$B$4,'Wellsfargo'!A:A,"&lt;="&amp;$D$4)</f>
+        <f>SUMIFS('Wellsfargo'!F:F,'Wellsfargo'!A:A,"&gt;="&amp;$B$4,'Wellsfargo'!A:A,"&lt;="&amp;$D$4)</f>
         <v/>
       </c>
       <c r="E10" s="15">
-        <f>SUMIFS('Wellsfargo'!F:F,'Wellsfargo'!A:A,"&gt;="&amp;$B$4,'Wellsfargo'!A:A,"&lt;="&amp;$D$4)</f>
-        <v/>
-      </c>
-      <c r="F10" s="15">
-        <f>C10-D10-E10</f>
+        <f>B10-C10-D10</f>
         <v/>
       </c>
     </row>
@@ -702,41 +676,49 @@
         </is>
       </c>
       <c r="B11" s="15">
-        <f>'Vyral'!B4</f>
+        <f>SUMIFS('Vyral'!D:D,'Vyral'!A:A,"&gt;="&amp;$B$4,'Vyral'!A:A,"&lt;="&amp;$D$4)</f>
         <v/>
       </c>
       <c r="C11" s="15">
-        <f>SUMIFS('Vyral'!D:D,'Vyral'!A:A,"&gt;="&amp;$B$4,'Vyral'!A:A,"&lt;="&amp;$D$4)</f>
+        <f>SUMIFS('Vyral'!E:E,'Vyral'!A:A,"&gt;="&amp;$B$4,'Vyral'!A:A,"&lt;="&amp;$D$4)</f>
         <v/>
       </c>
       <c r="D11" s="15">
-        <f>SUMIFS('Vyral'!E:E,'Vyral'!A:A,"&gt;="&amp;$B$4,'Vyral'!A:A,"&lt;="&amp;$D$4)</f>
+        <f>SUMIFS('Vyral'!F:F,'Vyral'!A:A,"&gt;="&amp;$B$4,'Vyral'!A:A,"&lt;="&amp;$D$4)</f>
         <v/>
       </c>
       <c r="E11" s="15">
-        <f>SUMIFS('Vyral'!F:F,'Vyral'!A:A,"&gt;="&amp;$B$4,'Vyral'!A:A,"&lt;="&amp;$D$4)</f>
-        <v/>
-      </c>
-      <c r="F11" s="15">
-        <f>C11-D11-E11</f>
+        <f>B11-C11-D11</f>
         <v/>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Total USD Bank Balance</t>
+          <t>USD Bank Totals</t>
         </is>
       </c>
       <c r="B13" s="16">
         <f>SUM(B8:B11)</f>
+        <v/>
+      </c>
+      <c r="C13" s="16">
+        <f>SUM(C8:C11)</f>
+        <v/>
+      </c>
+      <c r="D13" s="16">
+        <f>SUM(D8:D11)</f>
+        <v/>
+      </c>
+      <c r="E13" s="16">
+        <f>SUM(E8:E11)</f>
         <v/>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>GHS Bank Accounts (Ghana Cedis)</t>
+          <t>Selected Month - GHS Bank Accounts</t>
         </is>
       </c>
     </row>
@@ -748,27 +730,22 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>Current Balance (GHS)</t>
+          <t>Money In</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>Month In</t>
+          <t>Money Out</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>Month Out</t>
+          <t>Tax</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>Month Tax</t>
-        </is>
-      </c>
-      <c r="F17" s="5" t="inlineStr">
-        <is>
-          <t>Net Month Change</t>
+          <t>Net Flow</t>
         </is>
       </c>
     </row>
@@ -779,138 +756,2134 @@
         </is>
       </c>
       <c r="B18" s="9">
-        <f>'Ghana City'!B4</f>
+        <f>SUMIFS('Ghana City'!D:D,'Ghana City'!A:A,"&gt;="&amp;$B$4,'Ghana City'!A:A,"&lt;="&amp;$D$4)</f>
         <v/>
       </c>
       <c r="C18" s="9">
-        <f>SUMIFS('Ghana City'!D:D,'Ghana City'!A:A,"&gt;="&amp;$B$4,'Ghana City'!A:A,"&lt;="&amp;$D$4)</f>
+        <f>SUMIFS('Ghana City'!E:E,'Ghana City'!A:A,"&gt;="&amp;$B$4,'Ghana City'!A:A,"&lt;="&amp;$D$4)</f>
         <v/>
       </c>
       <c r="D18" s="9">
-        <f>SUMIFS('Ghana City'!E:E,'Ghana City'!A:A,"&gt;="&amp;$B$4,'Ghana City'!A:A,"&lt;="&amp;$D$4)</f>
+        <f>SUMIFS('Ghana City'!F:F,'Ghana City'!A:A,"&gt;="&amp;$B$4,'Ghana City'!A:A,"&lt;="&amp;$D$4)</f>
         <v/>
       </c>
       <c r="E18" s="9">
-        <f>SUMIFS('Ghana City'!F:F,'Ghana City'!A:A,"&gt;="&amp;$B$4,'Ghana City'!A:A,"&lt;="&amp;$D$4)</f>
-        <v/>
-      </c>
-      <c r="F18" s="9">
-        <f>C18-D18-E18</f>
-        <v/>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="4" t="inlineStr">
+        <f>B18-C18-D18</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>Credit Cards (USD Liabilities)</t>
+          <t>Selected Month - Credit Cards (USD)</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="5" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
         <is>
           <t>Card</t>
         </is>
       </c>
-      <c r="B24" s="5" t="inlineStr">
+      <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>Current Owed (USD)</t>
+          <t>Payments In</t>
         </is>
       </c>
-      <c r="C24" s="5" t="inlineStr">
+      <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>Month Payments</t>
+          <t>Spend Out</t>
         </is>
       </c>
-      <c r="D24" s="5" t="inlineStr">
+      <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>Month Spend</t>
+          <t>Tax</t>
         </is>
       </c>
-      <c r="E24" s="5" t="inlineStr">
-        <is>
-          <t>Month Tax</t>
-        </is>
-      </c>
-      <c r="F24" s="5" t="inlineStr">
+      <c r="E22" s="5" t="inlineStr">
         <is>
           <t>Net Owed Change</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="6" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="6" t="inlineStr">
         <is>
           <t>Credit Card 1</t>
         </is>
       </c>
-      <c r="B25" s="15">
-        <f>'Credit Card 1'!B4</f>
-        <v/>
-      </c>
-      <c r="C25" s="15">
+      <c r="B23" s="15">
         <f>SUMIFS('Credit Card 1'!D:D,'Credit Card 1'!A:A,"&gt;="&amp;$B$4,'Credit Card 1'!A:A,"&lt;="&amp;$D$4)</f>
         <v/>
       </c>
-      <c r="D25" s="15">
+      <c r="C23" s="15">
         <f>SUMIFS('Credit Card 1'!E:E,'Credit Card 1'!A:A,"&gt;="&amp;$B$4,'Credit Card 1'!A:A,"&lt;="&amp;$D$4)</f>
         <v/>
       </c>
-      <c r="E25" s="15">
+      <c r="D23" s="15">
         <f>SUMIFS('Credit Card 1'!F:F,'Credit Card 1'!A:A,"&gt;="&amp;$B$4,'Credit Card 1'!A:A,"&lt;="&amp;$D$4)</f>
         <v/>
       </c>
-      <c r="F25" s="15">
-        <f>D25+E25-C25</f>
-        <v/>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="6" t="inlineStr">
+      <c r="E23" s="15">
+        <f>C23+D23-B23</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="inlineStr">
         <is>
           <t>Credit Card 2</t>
         </is>
       </c>
-      <c r="B26" s="15">
-        <f>'Credit Card 2'!B4</f>
-        <v/>
-      </c>
-      <c r="C26" s="15">
+      <c r="B24" s="15">
         <f>SUMIFS('Credit Card 2'!D:D,'Credit Card 2'!A:A,"&gt;="&amp;$B$4,'Credit Card 2'!A:A,"&lt;="&amp;$D$4)</f>
         <v/>
       </c>
-      <c r="D26" s="15">
+      <c r="C24" s="15">
         <f>SUMIFS('Credit Card 2'!E:E,'Credit Card 2'!A:A,"&gt;="&amp;$B$4,'Credit Card 2'!A:A,"&lt;="&amp;$D$4)</f>
         <v/>
       </c>
-      <c r="E26" s="15">
+      <c r="D24" s="15">
         <f>SUMIFS('Credit Card 2'!F:F,'Credit Card 2'!A:A,"&gt;="&amp;$B$4,'Credit Card 2'!A:A,"&lt;="&amp;$D$4)</f>
         <v/>
       </c>
-      <c r="F26" s="15">
-        <f>D26+E26-C26</f>
+      <c r="E24" s="15">
+        <f>C24+D24-B24</f>
         <v/>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="2" t="inlineStr">
+      <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>Total Credit Card Owed (USD)</t>
+          <t>Monthly Timeline (Apr 2026 to Apr 2029)</t>
         </is>
       </c>
-      <c r="B28" s="16">
-        <f>SUM(B25:B26)</f>
-        <v/>
-      </c>
     </row>
     <row r="29">
-      <c r="A29" s="2" t="inlineStr">
+      <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>Net USD Position (Banks - Cards)</t>
+          <t>Month</t>
         </is>
       </c>
-      <c r="B29" s="16">
-        <f>B13-B28</f>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>USD In</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>USD Out</t>
+        </is>
+      </c>
+      <c r="D29" s="5" t="inlineStr">
+        <is>
+          <t>USD Tax</t>
+        </is>
+      </c>
+      <c r="E29" s="5" t="inlineStr">
+        <is>
+          <t>USD Net</t>
+        </is>
+      </c>
+      <c r="F29" s="5" t="inlineStr">
+        <is>
+          <t>GHS In</t>
+        </is>
+      </c>
+      <c r="G29" s="5" t="inlineStr">
+        <is>
+          <t>GHS Out</t>
+        </is>
+      </c>
+      <c r="H29" s="5" t="inlineStr">
+        <is>
+          <t>GHS Tax</t>
+        </is>
+      </c>
+      <c r="I29" s="5" t="inlineStr">
+        <is>
+          <t>GHS Net</t>
+        </is>
+      </c>
+      <c r="J29" s="5" t="inlineStr">
+        <is>
+          <t>CC Payments</t>
+        </is>
+      </c>
+      <c r="K29" s="5" t="inlineStr">
+        <is>
+          <t>CC Spend</t>
+        </is>
+      </c>
+      <c r="L29" s="5" t="inlineStr">
+        <is>
+          <t>CC Tax</t>
+        </is>
+      </c>
+      <c r="M29" s="5" t="inlineStr">
+        <is>
+          <t>CC Net Owed Change</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="19" t="n">
+        <v>46113</v>
+      </c>
+      <c r="B30" s="15">
+        <f>SUMIFS('Current'!D:D,'Current'!A:A,"&gt;="&amp;EOMONTH($A30,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A30,0)) + SUMIFS('Chase'!D:D,'Chase'!A:A,"&gt;="&amp;EOMONTH($A30,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A30,0)) + SUMIFS('Wellsfargo'!D:D,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A30,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A30,0)) + SUMIFS('Vyral'!D:D,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A30,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A30,0))</f>
+        <v/>
+      </c>
+      <c r="C30" s="15">
+        <f>SUMIFS('Current'!E:E,'Current'!A:A,"&gt;="&amp;EOMONTH($A30,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A30,0)) + SUMIFS('Chase'!E:E,'Chase'!A:A,"&gt;="&amp;EOMONTH($A30,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A30,0)) + SUMIFS('Wellsfargo'!E:E,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A30,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A30,0)) + SUMIFS('Vyral'!E:E,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A30,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A30,0))</f>
+        <v/>
+      </c>
+      <c r="D30" s="15">
+        <f>SUMIFS('Current'!F:F,'Current'!A:A,"&gt;="&amp;EOMONTH($A30,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A30,0)) + SUMIFS('Chase'!F:F,'Chase'!A:A,"&gt;="&amp;EOMONTH($A30,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A30,0)) + SUMIFS('Wellsfargo'!F:F,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A30,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A30,0)) + SUMIFS('Vyral'!F:F,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A30,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A30,0))</f>
+        <v/>
+      </c>
+      <c r="E30" s="15">
+        <f>B30-C30-D30</f>
+        <v/>
+      </c>
+      <c r="F30" s="9">
+        <f>SUMIFS('Ghana City'!D:D,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A30,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A30,0))</f>
+        <v/>
+      </c>
+      <c r="G30" s="9">
+        <f>SUMIFS('Ghana City'!E:E,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A30,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A30,0))</f>
+        <v/>
+      </c>
+      <c r="H30" s="9">
+        <f>SUMIFS('Ghana City'!F:F,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A30,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A30,0))</f>
+        <v/>
+      </c>
+      <c r="I30" s="9">
+        <f>F30-G30-H30</f>
+        <v/>
+      </c>
+      <c r="J30" s="15">
+        <f>SUMIFS('Credit Card 1'!D:D,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A30,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A30,0)) + SUMIFS('Credit Card 2'!D:D,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A30,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A30,0))</f>
+        <v/>
+      </c>
+      <c r="K30" s="15">
+        <f>SUMIFS('Credit Card 1'!E:E,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A30,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A30,0)) + SUMIFS('Credit Card 2'!E:E,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A30,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A30,0))</f>
+        <v/>
+      </c>
+      <c r="L30" s="15">
+        <f>SUMIFS('Credit Card 1'!F:F,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A30,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A30,0)) + SUMIFS('Credit Card 2'!F:F,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A30,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A30,0))</f>
+        <v/>
+      </c>
+      <c r="M30" s="15">
+        <f>K30+L30-J30</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="19" t="n">
+        <v>46143</v>
+      </c>
+      <c r="B31" s="15">
+        <f>SUMIFS('Current'!D:D,'Current'!A:A,"&gt;="&amp;EOMONTH($A31,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A31,0)) + SUMIFS('Chase'!D:D,'Chase'!A:A,"&gt;="&amp;EOMONTH($A31,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A31,0)) + SUMIFS('Wellsfargo'!D:D,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A31,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A31,0)) + SUMIFS('Vyral'!D:D,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A31,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A31,0))</f>
+        <v/>
+      </c>
+      <c r="C31" s="15">
+        <f>SUMIFS('Current'!E:E,'Current'!A:A,"&gt;="&amp;EOMONTH($A31,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A31,0)) + SUMIFS('Chase'!E:E,'Chase'!A:A,"&gt;="&amp;EOMONTH($A31,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A31,0)) + SUMIFS('Wellsfargo'!E:E,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A31,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A31,0)) + SUMIFS('Vyral'!E:E,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A31,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A31,0))</f>
+        <v/>
+      </c>
+      <c r="D31" s="15">
+        <f>SUMIFS('Current'!F:F,'Current'!A:A,"&gt;="&amp;EOMONTH($A31,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A31,0)) + SUMIFS('Chase'!F:F,'Chase'!A:A,"&gt;="&amp;EOMONTH($A31,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A31,0)) + SUMIFS('Wellsfargo'!F:F,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A31,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A31,0)) + SUMIFS('Vyral'!F:F,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A31,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A31,0))</f>
+        <v/>
+      </c>
+      <c r="E31" s="15">
+        <f>B31-C31-D31</f>
+        <v/>
+      </c>
+      <c r="F31" s="9">
+        <f>SUMIFS('Ghana City'!D:D,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A31,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A31,0))</f>
+        <v/>
+      </c>
+      <c r="G31" s="9">
+        <f>SUMIFS('Ghana City'!E:E,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A31,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A31,0))</f>
+        <v/>
+      </c>
+      <c r="H31" s="9">
+        <f>SUMIFS('Ghana City'!F:F,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A31,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A31,0))</f>
+        <v/>
+      </c>
+      <c r="I31" s="9">
+        <f>F31-G31-H31</f>
+        <v/>
+      </c>
+      <c r="J31" s="15">
+        <f>SUMIFS('Credit Card 1'!D:D,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A31,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A31,0)) + SUMIFS('Credit Card 2'!D:D,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A31,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A31,0))</f>
+        <v/>
+      </c>
+      <c r="K31" s="15">
+        <f>SUMIFS('Credit Card 1'!E:E,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A31,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A31,0)) + SUMIFS('Credit Card 2'!E:E,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A31,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A31,0))</f>
+        <v/>
+      </c>
+      <c r="L31" s="15">
+        <f>SUMIFS('Credit Card 1'!F:F,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A31,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A31,0)) + SUMIFS('Credit Card 2'!F:F,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A31,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A31,0))</f>
+        <v/>
+      </c>
+      <c r="M31" s="15">
+        <f>K31+L31-J31</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="19" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B32" s="15">
+        <f>SUMIFS('Current'!D:D,'Current'!A:A,"&gt;="&amp;EOMONTH($A32,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A32,0)) + SUMIFS('Chase'!D:D,'Chase'!A:A,"&gt;="&amp;EOMONTH($A32,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A32,0)) + SUMIFS('Wellsfargo'!D:D,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A32,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A32,0)) + SUMIFS('Vyral'!D:D,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A32,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A32,0))</f>
+        <v/>
+      </c>
+      <c r="C32" s="15">
+        <f>SUMIFS('Current'!E:E,'Current'!A:A,"&gt;="&amp;EOMONTH($A32,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A32,0)) + SUMIFS('Chase'!E:E,'Chase'!A:A,"&gt;="&amp;EOMONTH($A32,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A32,0)) + SUMIFS('Wellsfargo'!E:E,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A32,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A32,0)) + SUMIFS('Vyral'!E:E,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A32,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A32,0))</f>
+        <v/>
+      </c>
+      <c r="D32" s="15">
+        <f>SUMIFS('Current'!F:F,'Current'!A:A,"&gt;="&amp;EOMONTH($A32,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A32,0)) + SUMIFS('Chase'!F:F,'Chase'!A:A,"&gt;="&amp;EOMONTH($A32,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A32,0)) + SUMIFS('Wellsfargo'!F:F,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A32,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A32,0)) + SUMIFS('Vyral'!F:F,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A32,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A32,0))</f>
+        <v/>
+      </c>
+      <c r="E32" s="15">
+        <f>B32-C32-D32</f>
+        <v/>
+      </c>
+      <c r="F32" s="9">
+        <f>SUMIFS('Ghana City'!D:D,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A32,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A32,0))</f>
+        <v/>
+      </c>
+      <c r="G32" s="9">
+        <f>SUMIFS('Ghana City'!E:E,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A32,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A32,0))</f>
+        <v/>
+      </c>
+      <c r="H32" s="9">
+        <f>SUMIFS('Ghana City'!F:F,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A32,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A32,0))</f>
+        <v/>
+      </c>
+      <c r="I32" s="9">
+        <f>F32-G32-H32</f>
+        <v/>
+      </c>
+      <c r="J32" s="15">
+        <f>SUMIFS('Credit Card 1'!D:D,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A32,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A32,0)) + SUMIFS('Credit Card 2'!D:D,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A32,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A32,0))</f>
+        <v/>
+      </c>
+      <c r="K32" s="15">
+        <f>SUMIFS('Credit Card 1'!E:E,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A32,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A32,0)) + SUMIFS('Credit Card 2'!E:E,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A32,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A32,0))</f>
+        <v/>
+      </c>
+      <c r="L32" s="15">
+        <f>SUMIFS('Credit Card 1'!F:F,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A32,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A32,0)) + SUMIFS('Credit Card 2'!F:F,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A32,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A32,0))</f>
+        <v/>
+      </c>
+      <c r="M32" s="15">
+        <f>K32+L32-J32</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="19" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B33" s="15">
+        <f>SUMIFS('Current'!D:D,'Current'!A:A,"&gt;="&amp;EOMONTH($A33,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A33,0)) + SUMIFS('Chase'!D:D,'Chase'!A:A,"&gt;="&amp;EOMONTH($A33,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A33,0)) + SUMIFS('Wellsfargo'!D:D,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A33,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A33,0)) + SUMIFS('Vyral'!D:D,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A33,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A33,0))</f>
+        <v/>
+      </c>
+      <c r="C33" s="15">
+        <f>SUMIFS('Current'!E:E,'Current'!A:A,"&gt;="&amp;EOMONTH($A33,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A33,0)) + SUMIFS('Chase'!E:E,'Chase'!A:A,"&gt;="&amp;EOMONTH($A33,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A33,0)) + SUMIFS('Wellsfargo'!E:E,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A33,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A33,0)) + SUMIFS('Vyral'!E:E,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A33,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A33,0))</f>
+        <v/>
+      </c>
+      <c r="D33" s="15">
+        <f>SUMIFS('Current'!F:F,'Current'!A:A,"&gt;="&amp;EOMONTH($A33,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A33,0)) + SUMIFS('Chase'!F:F,'Chase'!A:A,"&gt;="&amp;EOMONTH($A33,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A33,0)) + SUMIFS('Wellsfargo'!F:F,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A33,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A33,0)) + SUMIFS('Vyral'!F:F,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A33,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A33,0))</f>
+        <v/>
+      </c>
+      <c r="E33" s="15">
+        <f>B33-C33-D33</f>
+        <v/>
+      </c>
+      <c r="F33" s="9">
+        <f>SUMIFS('Ghana City'!D:D,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A33,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A33,0))</f>
+        <v/>
+      </c>
+      <c r="G33" s="9">
+        <f>SUMIFS('Ghana City'!E:E,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A33,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A33,0))</f>
+        <v/>
+      </c>
+      <c r="H33" s="9">
+        <f>SUMIFS('Ghana City'!F:F,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A33,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A33,0))</f>
+        <v/>
+      </c>
+      <c r="I33" s="9">
+        <f>F33-G33-H33</f>
+        <v/>
+      </c>
+      <c r="J33" s="15">
+        <f>SUMIFS('Credit Card 1'!D:D,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A33,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A33,0)) + SUMIFS('Credit Card 2'!D:D,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A33,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A33,0))</f>
+        <v/>
+      </c>
+      <c r="K33" s="15">
+        <f>SUMIFS('Credit Card 1'!E:E,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A33,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A33,0)) + SUMIFS('Credit Card 2'!E:E,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A33,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A33,0))</f>
+        <v/>
+      </c>
+      <c r="L33" s="15">
+        <f>SUMIFS('Credit Card 1'!F:F,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A33,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A33,0)) + SUMIFS('Credit Card 2'!F:F,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A33,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A33,0))</f>
+        <v/>
+      </c>
+      <c r="M33" s="15">
+        <f>K33+L33-J33</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="19" t="n">
+        <v>46235</v>
+      </c>
+      <c r="B34" s="15">
+        <f>SUMIFS('Current'!D:D,'Current'!A:A,"&gt;="&amp;EOMONTH($A34,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A34,0)) + SUMIFS('Chase'!D:D,'Chase'!A:A,"&gt;="&amp;EOMONTH($A34,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A34,0)) + SUMIFS('Wellsfargo'!D:D,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A34,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A34,0)) + SUMIFS('Vyral'!D:D,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A34,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A34,0))</f>
+        <v/>
+      </c>
+      <c r="C34" s="15">
+        <f>SUMIFS('Current'!E:E,'Current'!A:A,"&gt;="&amp;EOMONTH($A34,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A34,0)) + SUMIFS('Chase'!E:E,'Chase'!A:A,"&gt;="&amp;EOMONTH($A34,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A34,0)) + SUMIFS('Wellsfargo'!E:E,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A34,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A34,0)) + SUMIFS('Vyral'!E:E,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A34,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A34,0))</f>
+        <v/>
+      </c>
+      <c r="D34" s="15">
+        <f>SUMIFS('Current'!F:F,'Current'!A:A,"&gt;="&amp;EOMONTH($A34,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A34,0)) + SUMIFS('Chase'!F:F,'Chase'!A:A,"&gt;="&amp;EOMONTH($A34,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A34,0)) + SUMIFS('Wellsfargo'!F:F,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A34,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A34,0)) + SUMIFS('Vyral'!F:F,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A34,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A34,0))</f>
+        <v/>
+      </c>
+      <c r="E34" s="15">
+        <f>B34-C34-D34</f>
+        <v/>
+      </c>
+      <c r="F34" s="9">
+        <f>SUMIFS('Ghana City'!D:D,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A34,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A34,0))</f>
+        <v/>
+      </c>
+      <c r="G34" s="9">
+        <f>SUMIFS('Ghana City'!E:E,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A34,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A34,0))</f>
+        <v/>
+      </c>
+      <c r="H34" s="9">
+        <f>SUMIFS('Ghana City'!F:F,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A34,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A34,0))</f>
+        <v/>
+      </c>
+      <c r="I34" s="9">
+        <f>F34-G34-H34</f>
+        <v/>
+      </c>
+      <c r="J34" s="15">
+        <f>SUMIFS('Credit Card 1'!D:D,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A34,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A34,0)) + SUMIFS('Credit Card 2'!D:D,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A34,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A34,0))</f>
+        <v/>
+      </c>
+      <c r="K34" s="15">
+        <f>SUMIFS('Credit Card 1'!E:E,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A34,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A34,0)) + SUMIFS('Credit Card 2'!E:E,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A34,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A34,0))</f>
+        <v/>
+      </c>
+      <c r="L34" s="15">
+        <f>SUMIFS('Credit Card 1'!F:F,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A34,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A34,0)) + SUMIFS('Credit Card 2'!F:F,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A34,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A34,0))</f>
+        <v/>
+      </c>
+      <c r="M34" s="15">
+        <f>K34+L34-J34</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="19" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B35" s="15">
+        <f>SUMIFS('Current'!D:D,'Current'!A:A,"&gt;="&amp;EOMONTH($A35,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A35,0)) + SUMIFS('Chase'!D:D,'Chase'!A:A,"&gt;="&amp;EOMONTH($A35,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A35,0)) + SUMIFS('Wellsfargo'!D:D,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A35,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A35,0)) + SUMIFS('Vyral'!D:D,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A35,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A35,0))</f>
+        <v/>
+      </c>
+      <c r="C35" s="15">
+        <f>SUMIFS('Current'!E:E,'Current'!A:A,"&gt;="&amp;EOMONTH($A35,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A35,0)) + SUMIFS('Chase'!E:E,'Chase'!A:A,"&gt;="&amp;EOMONTH($A35,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A35,0)) + SUMIFS('Wellsfargo'!E:E,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A35,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A35,0)) + SUMIFS('Vyral'!E:E,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A35,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A35,0))</f>
+        <v/>
+      </c>
+      <c r="D35" s="15">
+        <f>SUMIFS('Current'!F:F,'Current'!A:A,"&gt;="&amp;EOMONTH($A35,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A35,0)) + SUMIFS('Chase'!F:F,'Chase'!A:A,"&gt;="&amp;EOMONTH($A35,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A35,0)) + SUMIFS('Wellsfargo'!F:F,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A35,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A35,0)) + SUMIFS('Vyral'!F:F,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A35,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A35,0))</f>
+        <v/>
+      </c>
+      <c r="E35" s="15">
+        <f>B35-C35-D35</f>
+        <v/>
+      </c>
+      <c r="F35" s="9">
+        <f>SUMIFS('Ghana City'!D:D,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A35,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A35,0))</f>
+        <v/>
+      </c>
+      <c r="G35" s="9">
+        <f>SUMIFS('Ghana City'!E:E,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A35,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A35,0))</f>
+        <v/>
+      </c>
+      <c r="H35" s="9">
+        <f>SUMIFS('Ghana City'!F:F,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A35,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A35,0))</f>
+        <v/>
+      </c>
+      <c r="I35" s="9">
+        <f>F35-G35-H35</f>
+        <v/>
+      </c>
+      <c r="J35" s="15">
+        <f>SUMIFS('Credit Card 1'!D:D,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A35,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A35,0)) + SUMIFS('Credit Card 2'!D:D,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A35,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A35,0))</f>
+        <v/>
+      </c>
+      <c r="K35" s="15">
+        <f>SUMIFS('Credit Card 1'!E:E,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A35,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A35,0)) + SUMIFS('Credit Card 2'!E:E,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A35,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A35,0))</f>
+        <v/>
+      </c>
+      <c r="L35" s="15">
+        <f>SUMIFS('Credit Card 1'!F:F,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A35,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A35,0)) + SUMIFS('Credit Card 2'!F:F,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A35,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A35,0))</f>
+        <v/>
+      </c>
+      <c r="M35" s="15">
+        <f>K35+L35-J35</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="19" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B36" s="15">
+        <f>SUMIFS('Current'!D:D,'Current'!A:A,"&gt;="&amp;EOMONTH($A36,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A36,0)) + SUMIFS('Chase'!D:D,'Chase'!A:A,"&gt;="&amp;EOMONTH($A36,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A36,0)) + SUMIFS('Wellsfargo'!D:D,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A36,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A36,0)) + SUMIFS('Vyral'!D:D,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A36,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A36,0))</f>
+        <v/>
+      </c>
+      <c r="C36" s="15">
+        <f>SUMIFS('Current'!E:E,'Current'!A:A,"&gt;="&amp;EOMONTH($A36,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A36,0)) + SUMIFS('Chase'!E:E,'Chase'!A:A,"&gt;="&amp;EOMONTH($A36,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A36,0)) + SUMIFS('Wellsfargo'!E:E,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A36,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A36,0)) + SUMIFS('Vyral'!E:E,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A36,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A36,0))</f>
+        <v/>
+      </c>
+      <c r="D36" s="15">
+        <f>SUMIFS('Current'!F:F,'Current'!A:A,"&gt;="&amp;EOMONTH($A36,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A36,0)) + SUMIFS('Chase'!F:F,'Chase'!A:A,"&gt;="&amp;EOMONTH($A36,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A36,0)) + SUMIFS('Wellsfargo'!F:F,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A36,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A36,0)) + SUMIFS('Vyral'!F:F,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A36,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A36,0))</f>
+        <v/>
+      </c>
+      <c r="E36" s="15">
+        <f>B36-C36-D36</f>
+        <v/>
+      </c>
+      <c r="F36" s="9">
+        <f>SUMIFS('Ghana City'!D:D,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A36,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A36,0))</f>
+        <v/>
+      </c>
+      <c r="G36" s="9">
+        <f>SUMIFS('Ghana City'!E:E,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A36,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A36,0))</f>
+        <v/>
+      </c>
+      <c r="H36" s="9">
+        <f>SUMIFS('Ghana City'!F:F,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A36,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A36,0))</f>
+        <v/>
+      </c>
+      <c r="I36" s="9">
+        <f>F36-G36-H36</f>
+        <v/>
+      </c>
+      <c r="J36" s="15">
+        <f>SUMIFS('Credit Card 1'!D:D,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A36,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A36,0)) + SUMIFS('Credit Card 2'!D:D,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A36,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A36,0))</f>
+        <v/>
+      </c>
+      <c r="K36" s="15">
+        <f>SUMIFS('Credit Card 1'!E:E,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A36,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A36,0)) + SUMIFS('Credit Card 2'!E:E,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A36,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A36,0))</f>
+        <v/>
+      </c>
+      <c r="L36" s="15">
+        <f>SUMIFS('Credit Card 1'!F:F,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A36,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A36,0)) + SUMIFS('Credit Card 2'!F:F,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A36,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A36,0))</f>
+        <v/>
+      </c>
+      <c r="M36" s="15">
+        <f>K36+L36-J36</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="19" t="n">
+        <v>46327</v>
+      </c>
+      <c r="B37" s="15">
+        <f>SUMIFS('Current'!D:D,'Current'!A:A,"&gt;="&amp;EOMONTH($A37,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A37,0)) + SUMIFS('Chase'!D:D,'Chase'!A:A,"&gt;="&amp;EOMONTH($A37,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A37,0)) + SUMIFS('Wellsfargo'!D:D,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A37,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A37,0)) + SUMIFS('Vyral'!D:D,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A37,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A37,0))</f>
+        <v/>
+      </c>
+      <c r="C37" s="15">
+        <f>SUMIFS('Current'!E:E,'Current'!A:A,"&gt;="&amp;EOMONTH($A37,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A37,0)) + SUMIFS('Chase'!E:E,'Chase'!A:A,"&gt;="&amp;EOMONTH($A37,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A37,0)) + SUMIFS('Wellsfargo'!E:E,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A37,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A37,0)) + SUMIFS('Vyral'!E:E,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A37,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A37,0))</f>
+        <v/>
+      </c>
+      <c r="D37" s="15">
+        <f>SUMIFS('Current'!F:F,'Current'!A:A,"&gt;="&amp;EOMONTH($A37,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A37,0)) + SUMIFS('Chase'!F:F,'Chase'!A:A,"&gt;="&amp;EOMONTH($A37,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A37,0)) + SUMIFS('Wellsfargo'!F:F,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A37,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A37,0)) + SUMIFS('Vyral'!F:F,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A37,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A37,0))</f>
+        <v/>
+      </c>
+      <c r="E37" s="15">
+        <f>B37-C37-D37</f>
+        <v/>
+      </c>
+      <c r="F37" s="9">
+        <f>SUMIFS('Ghana City'!D:D,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A37,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A37,0))</f>
+        <v/>
+      </c>
+      <c r="G37" s="9">
+        <f>SUMIFS('Ghana City'!E:E,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A37,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A37,0))</f>
+        <v/>
+      </c>
+      <c r="H37" s="9">
+        <f>SUMIFS('Ghana City'!F:F,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A37,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A37,0))</f>
+        <v/>
+      </c>
+      <c r="I37" s="9">
+        <f>F37-G37-H37</f>
+        <v/>
+      </c>
+      <c r="J37" s="15">
+        <f>SUMIFS('Credit Card 1'!D:D,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A37,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A37,0)) + SUMIFS('Credit Card 2'!D:D,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A37,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A37,0))</f>
+        <v/>
+      </c>
+      <c r="K37" s="15">
+        <f>SUMIFS('Credit Card 1'!E:E,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A37,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A37,0)) + SUMIFS('Credit Card 2'!E:E,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A37,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A37,0))</f>
+        <v/>
+      </c>
+      <c r="L37" s="15">
+        <f>SUMIFS('Credit Card 1'!F:F,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A37,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A37,0)) + SUMIFS('Credit Card 2'!F:F,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A37,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A37,0))</f>
+        <v/>
+      </c>
+      <c r="M37" s="15">
+        <f>K37+L37-J37</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="19" t="n">
+        <v>46357</v>
+      </c>
+      <c r="B38" s="15">
+        <f>SUMIFS('Current'!D:D,'Current'!A:A,"&gt;="&amp;EOMONTH($A38,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A38,0)) + SUMIFS('Chase'!D:D,'Chase'!A:A,"&gt;="&amp;EOMONTH($A38,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A38,0)) + SUMIFS('Wellsfargo'!D:D,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A38,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A38,0)) + SUMIFS('Vyral'!D:D,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A38,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A38,0))</f>
+        <v/>
+      </c>
+      <c r="C38" s="15">
+        <f>SUMIFS('Current'!E:E,'Current'!A:A,"&gt;="&amp;EOMONTH($A38,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A38,0)) + SUMIFS('Chase'!E:E,'Chase'!A:A,"&gt;="&amp;EOMONTH($A38,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A38,0)) + SUMIFS('Wellsfargo'!E:E,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A38,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A38,0)) + SUMIFS('Vyral'!E:E,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A38,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A38,0))</f>
+        <v/>
+      </c>
+      <c r="D38" s="15">
+        <f>SUMIFS('Current'!F:F,'Current'!A:A,"&gt;="&amp;EOMONTH($A38,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A38,0)) + SUMIFS('Chase'!F:F,'Chase'!A:A,"&gt;="&amp;EOMONTH($A38,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A38,0)) + SUMIFS('Wellsfargo'!F:F,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A38,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A38,0)) + SUMIFS('Vyral'!F:F,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A38,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A38,0))</f>
+        <v/>
+      </c>
+      <c r="E38" s="15">
+        <f>B38-C38-D38</f>
+        <v/>
+      </c>
+      <c r="F38" s="9">
+        <f>SUMIFS('Ghana City'!D:D,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A38,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A38,0))</f>
+        <v/>
+      </c>
+      <c r="G38" s="9">
+        <f>SUMIFS('Ghana City'!E:E,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A38,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A38,0))</f>
+        <v/>
+      </c>
+      <c r="H38" s="9">
+        <f>SUMIFS('Ghana City'!F:F,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A38,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A38,0))</f>
+        <v/>
+      </c>
+      <c r="I38" s="9">
+        <f>F38-G38-H38</f>
+        <v/>
+      </c>
+      <c r="J38" s="15">
+        <f>SUMIFS('Credit Card 1'!D:D,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A38,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A38,0)) + SUMIFS('Credit Card 2'!D:D,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A38,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A38,0))</f>
+        <v/>
+      </c>
+      <c r="K38" s="15">
+        <f>SUMIFS('Credit Card 1'!E:E,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A38,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A38,0)) + SUMIFS('Credit Card 2'!E:E,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A38,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A38,0))</f>
+        <v/>
+      </c>
+      <c r="L38" s="15">
+        <f>SUMIFS('Credit Card 1'!F:F,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A38,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A38,0)) + SUMIFS('Credit Card 2'!F:F,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A38,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A38,0))</f>
+        <v/>
+      </c>
+      <c r="M38" s="15">
+        <f>K38+L38-J38</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="19" t="n">
+        <v>46388</v>
+      </c>
+      <c r="B39" s="15">
+        <f>SUMIFS('Current'!D:D,'Current'!A:A,"&gt;="&amp;EOMONTH($A39,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A39,0)) + SUMIFS('Chase'!D:D,'Chase'!A:A,"&gt;="&amp;EOMONTH($A39,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A39,0)) + SUMIFS('Wellsfargo'!D:D,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A39,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A39,0)) + SUMIFS('Vyral'!D:D,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A39,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A39,0))</f>
+        <v/>
+      </c>
+      <c r="C39" s="15">
+        <f>SUMIFS('Current'!E:E,'Current'!A:A,"&gt;="&amp;EOMONTH($A39,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A39,0)) + SUMIFS('Chase'!E:E,'Chase'!A:A,"&gt;="&amp;EOMONTH($A39,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A39,0)) + SUMIFS('Wellsfargo'!E:E,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A39,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A39,0)) + SUMIFS('Vyral'!E:E,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A39,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A39,0))</f>
+        <v/>
+      </c>
+      <c r="D39" s="15">
+        <f>SUMIFS('Current'!F:F,'Current'!A:A,"&gt;="&amp;EOMONTH($A39,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A39,0)) + SUMIFS('Chase'!F:F,'Chase'!A:A,"&gt;="&amp;EOMONTH($A39,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A39,0)) + SUMIFS('Wellsfargo'!F:F,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A39,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A39,0)) + SUMIFS('Vyral'!F:F,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A39,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A39,0))</f>
+        <v/>
+      </c>
+      <c r="E39" s="15">
+        <f>B39-C39-D39</f>
+        <v/>
+      </c>
+      <c r="F39" s="9">
+        <f>SUMIFS('Ghana City'!D:D,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A39,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A39,0))</f>
+        <v/>
+      </c>
+      <c r="G39" s="9">
+        <f>SUMIFS('Ghana City'!E:E,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A39,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A39,0))</f>
+        <v/>
+      </c>
+      <c r="H39" s="9">
+        <f>SUMIFS('Ghana City'!F:F,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A39,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A39,0))</f>
+        <v/>
+      </c>
+      <c r="I39" s="9">
+        <f>F39-G39-H39</f>
+        <v/>
+      </c>
+      <c r="J39" s="15">
+        <f>SUMIFS('Credit Card 1'!D:D,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A39,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A39,0)) + SUMIFS('Credit Card 2'!D:D,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A39,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A39,0))</f>
+        <v/>
+      </c>
+      <c r="K39" s="15">
+        <f>SUMIFS('Credit Card 1'!E:E,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A39,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A39,0)) + SUMIFS('Credit Card 2'!E:E,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A39,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A39,0))</f>
+        <v/>
+      </c>
+      <c r="L39" s="15">
+        <f>SUMIFS('Credit Card 1'!F:F,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A39,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A39,0)) + SUMIFS('Credit Card 2'!F:F,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A39,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A39,0))</f>
+        <v/>
+      </c>
+      <c r="M39" s="15">
+        <f>K39+L39-J39</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="19" t="n">
+        <v>46419</v>
+      </c>
+      <c r="B40" s="15">
+        <f>SUMIFS('Current'!D:D,'Current'!A:A,"&gt;="&amp;EOMONTH($A40,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A40,0)) + SUMIFS('Chase'!D:D,'Chase'!A:A,"&gt;="&amp;EOMONTH($A40,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A40,0)) + SUMIFS('Wellsfargo'!D:D,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A40,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A40,0)) + SUMIFS('Vyral'!D:D,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A40,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A40,0))</f>
+        <v/>
+      </c>
+      <c r="C40" s="15">
+        <f>SUMIFS('Current'!E:E,'Current'!A:A,"&gt;="&amp;EOMONTH($A40,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A40,0)) + SUMIFS('Chase'!E:E,'Chase'!A:A,"&gt;="&amp;EOMONTH($A40,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A40,0)) + SUMIFS('Wellsfargo'!E:E,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A40,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A40,0)) + SUMIFS('Vyral'!E:E,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A40,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A40,0))</f>
+        <v/>
+      </c>
+      <c r="D40" s="15">
+        <f>SUMIFS('Current'!F:F,'Current'!A:A,"&gt;="&amp;EOMONTH($A40,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A40,0)) + SUMIFS('Chase'!F:F,'Chase'!A:A,"&gt;="&amp;EOMONTH($A40,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A40,0)) + SUMIFS('Wellsfargo'!F:F,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A40,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A40,0)) + SUMIFS('Vyral'!F:F,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A40,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A40,0))</f>
+        <v/>
+      </c>
+      <c r="E40" s="15">
+        <f>B40-C40-D40</f>
+        <v/>
+      </c>
+      <c r="F40" s="9">
+        <f>SUMIFS('Ghana City'!D:D,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A40,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A40,0))</f>
+        <v/>
+      </c>
+      <c r="G40" s="9">
+        <f>SUMIFS('Ghana City'!E:E,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A40,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A40,0))</f>
+        <v/>
+      </c>
+      <c r="H40" s="9">
+        <f>SUMIFS('Ghana City'!F:F,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A40,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A40,0))</f>
+        <v/>
+      </c>
+      <c r="I40" s="9">
+        <f>F40-G40-H40</f>
+        <v/>
+      </c>
+      <c r="J40" s="15">
+        <f>SUMIFS('Credit Card 1'!D:D,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A40,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A40,0)) + SUMIFS('Credit Card 2'!D:D,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A40,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A40,0))</f>
+        <v/>
+      </c>
+      <c r="K40" s="15">
+        <f>SUMIFS('Credit Card 1'!E:E,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A40,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A40,0)) + SUMIFS('Credit Card 2'!E:E,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A40,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A40,0))</f>
+        <v/>
+      </c>
+      <c r="L40" s="15">
+        <f>SUMIFS('Credit Card 1'!F:F,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A40,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A40,0)) + SUMIFS('Credit Card 2'!F:F,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A40,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A40,0))</f>
+        <v/>
+      </c>
+      <c r="M40" s="15">
+        <f>K40+L40-J40</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="19" t="n">
+        <v>46447</v>
+      </c>
+      <c r="B41" s="15">
+        <f>SUMIFS('Current'!D:D,'Current'!A:A,"&gt;="&amp;EOMONTH($A41,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A41,0)) + SUMIFS('Chase'!D:D,'Chase'!A:A,"&gt;="&amp;EOMONTH($A41,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A41,0)) + SUMIFS('Wellsfargo'!D:D,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A41,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A41,0)) + SUMIFS('Vyral'!D:D,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A41,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A41,0))</f>
+        <v/>
+      </c>
+      <c r="C41" s="15">
+        <f>SUMIFS('Current'!E:E,'Current'!A:A,"&gt;="&amp;EOMONTH($A41,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A41,0)) + SUMIFS('Chase'!E:E,'Chase'!A:A,"&gt;="&amp;EOMONTH($A41,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A41,0)) + SUMIFS('Wellsfargo'!E:E,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A41,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A41,0)) + SUMIFS('Vyral'!E:E,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A41,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A41,0))</f>
+        <v/>
+      </c>
+      <c r="D41" s="15">
+        <f>SUMIFS('Current'!F:F,'Current'!A:A,"&gt;="&amp;EOMONTH($A41,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A41,0)) + SUMIFS('Chase'!F:F,'Chase'!A:A,"&gt;="&amp;EOMONTH($A41,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A41,0)) + SUMIFS('Wellsfargo'!F:F,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A41,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A41,0)) + SUMIFS('Vyral'!F:F,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A41,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A41,0))</f>
+        <v/>
+      </c>
+      <c r="E41" s="15">
+        <f>B41-C41-D41</f>
+        <v/>
+      </c>
+      <c r="F41" s="9">
+        <f>SUMIFS('Ghana City'!D:D,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A41,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A41,0))</f>
+        <v/>
+      </c>
+      <c r="G41" s="9">
+        <f>SUMIFS('Ghana City'!E:E,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A41,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A41,0))</f>
+        <v/>
+      </c>
+      <c r="H41" s="9">
+        <f>SUMIFS('Ghana City'!F:F,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A41,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A41,0))</f>
+        <v/>
+      </c>
+      <c r="I41" s="9">
+        <f>F41-G41-H41</f>
+        <v/>
+      </c>
+      <c r="J41" s="15">
+        <f>SUMIFS('Credit Card 1'!D:D,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A41,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A41,0)) + SUMIFS('Credit Card 2'!D:D,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A41,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A41,0))</f>
+        <v/>
+      </c>
+      <c r="K41" s="15">
+        <f>SUMIFS('Credit Card 1'!E:E,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A41,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A41,0)) + SUMIFS('Credit Card 2'!E:E,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A41,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A41,0))</f>
+        <v/>
+      </c>
+      <c r="L41" s="15">
+        <f>SUMIFS('Credit Card 1'!F:F,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A41,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A41,0)) + SUMIFS('Credit Card 2'!F:F,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A41,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A41,0))</f>
+        <v/>
+      </c>
+      <c r="M41" s="15">
+        <f>K41+L41-J41</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="19" t="n">
+        <v>46478</v>
+      </c>
+      <c r="B42" s="15">
+        <f>SUMIFS('Current'!D:D,'Current'!A:A,"&gt;="&amp;EOMONTH($A42,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A42,0)) + SUMIFS('Chase'!D:D,'Chase'!A:A,"&gt;="&amp;EOMONTH($A42,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A42,0)) + SUMIFS('Wellsfargo'!D:D,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A42,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A42,0)) + SUMIFS('Vyral'!D:D,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A42,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A42,0))</f>
+        <v/>
+      </c>
+      <c r="C42" s="15">
+        <f>SUMIFS('Current'!E:E,'Current'!A:A,"&gt;="&amp;EOMONTH($A42,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A42,0)) + SUMIFS('Chase'!E:E,'Chase'!A:A,"&gt;="&amp;EOMONTH($A42,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A42,0)) + SUMIFS('Wellsfargo'!E:E,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A42,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A42,0)) + SUMIFS('Vyral'!E:E,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A42,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A42,0))</f>
+        <v/>
+      </c>
+      <c r="D42" s="15">
+        <f>SUMIFS('Current'!F:F,'Current'!A:A,"&gt;="&amp;EOMONTH($A42,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A42,0)) + SUMIFS('Chase'!F:F,'Chase'!A:A,"&gt;="&amp;EOMONTH($A42,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A42,0)) + SUMIFS('Wellsfargo'!F:F,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A42,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A42,0)) + SUMIFS('Vyral'!F:F,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A42,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A42,0))</f>
+        <v/>
+      </c>
+      <c r="E42" s="15">
+        <f>B42-C42-D42</f>
+        <v/>
+      </c>
+      <c r="F42" s="9">
+        <f>SUMIFS('Ghana City'!D:D,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A42,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A42,0))</f>
+        <v/>
+      </c>
+      <c r="G42" s="9">
+        <f>SUMIFS('Ghana City'!E:E,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A42,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A42,0))</f>
+        <v/>
+      </c>
+      <c r="H42" s="9">
+        <f>SUMIFS('Ghana City'!F:F,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A42,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A42,0))</f>
+        <v/>
+      </c>
+      <c r="I42" s="9">
+        <f>F42-G42-H42</f>
+        <v/>
+      </c>
+      <c r="J42" s="15">
+        <f>SUMIFS('Credit Card 1'!D:D,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A42,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A42,0)) + SUMIFS('Credit Card 2'!D:D,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A42,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A42,0))</f>
+        <v/>
+      </c>
+      <c r="K42" s="15">
+        <f>SUMIFS('Credit Card 1'!E:E,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A42,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A42,0)) + SUMIFS('Credit Card 2'!E:E,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A42,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A42,0))</f>
+        <v/>
+      </c>
+      <c r="L42" s="15">
+        <f>SUMIFS('Credit Card 1'!F:F,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A42,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A42,0)) + SUMIFS('Credit Card 2'!F:F,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A42,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A42,0))</f>
+        <v/>
+      </c>
+      <c r="M42" s="15">
+        <f>K42+L42-J42</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="19" t="n">
+        <v>46508</v>
+      </c>
+      <c r="B43" s="15">
+        <f>SUMIFS('Current'!D:D,'Current'!A:A,"&gt;="&amp;EOMONTH($A43,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A43,0)) + SUMIFS('Chase'!D:D,'Chase'!A:A,"&gt;="&amp;EOMONTH($A43,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A43,0)) + SUMIFS('Wellsfargo'!D:D,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A43,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A43,0)) + SUMIFS('Vyral'!D:D,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A43,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A43,0))</f>
+        <v/>
+      </c>
+      <c r="C43" s="15">
+        <f>SUMIFS('Current'!E:E,'Current'!A:A,"&gt;="&amp;EOMONTH($A43,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A43,0)) + SUMIFS('Chase'!E:E,'Chase'!A:A,"&gt;="&amp;EOMONTH($A43,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A43,0)) + SUMIFS('Wellsfargo'!E:E,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A43,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A43,0)) + SUMIFS('Vyral'!E:E,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A43,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A43,0))</f>
+        <v/>
+      </c>
+      <c r="D43" s="15">
+        <f>SUMIFS('Current'!F:F,'Current'!A:A,"&gt;="&amp;EOMONTH($A43,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A43,0)) + SUMIFS('Chase'!F:F,'Chase'!A:A,"&gt;="&amp;EOMONTH($A43,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A43,0)) + SUMIFS('Wellsfargo'!F:F,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A43,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A43,0)) + SUMIFS('Vyral'!F:F,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A43,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A43,0))</f>
+        <v/>
+      </c>
+      <c r="E43" s="15">
+        <f>B43-C43-D43</f>
+        <v/>
+      </c>
+      <c r="F43" s="9">
+        <f>SUMIFS('Ghana City'!D:D,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A43,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A43,0))</f>
+        <v/>
+      </c>
+      <c r="G43" s="9">
+        <f>SUMIFS('Ghana City'!E:E,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A43,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A43,0))</f>
+        <v/>
+      </c>
+      <c r="H43" s="9">
+        <f>SUMIFS('Ghana City'!F:F,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A43,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A43,0))</f>
+        <v/>
+      </c>
+      <c r="I43" s="9">
+        <f>F43-G43-H43</f>
+        <v/>
+      </c>
+      <c r="J43" s="15">
+        <f>SUMIFS('Credit Card 1'!D:D,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A43,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A43,0)) + SUMIFS('Credit Card 2'!D:D,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A43,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A43,0))</f>
+        <v/>
+      </c>
+      <c r="K43" s="15">
+        <f>SUMIFS('Credit Card 1'!E:E,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A43,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A43,0)) + SUMIFS('Credit Card 2'!E:E,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A43,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A43,0))</f>
+        <v/>
+      </c>
+      <c r="L43" s="15">
+        <f>SUMIFS('Credit Card 1'!F:F,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A43,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A43,0)) + SUMIFS('Credit Card 2'!F:F,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A43,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A43,0))</f>
+        <v/>
+      </c>
+      <c r="M43" s="15">
+        <f>K43+L43-J43</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="19" t="n">
+        <v>46539</v>
+      </c>
+      <c r="B44" s="15">
+        <f>SUMIFS('Current'!D:D,'Current'!A:A,"&gt;="&amp;EOMONTH($A44,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A44,0)) + SUMIFS('Chase'!D:D,'Chase'!A:A,"&gt;="&amp;EOMONTH($A44,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A44,0)) + SUMIFS('Wellsfargo'!D:D,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A44,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A44,0)) + SUMIFS('Vyral'!D:D,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A44,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A44,0))</f>
+        <v/>
+      </c>
+      <c r="C44" s="15">
+        <f>SUMIFS('Current'!E:E,'Current'!A:A,"&gt;="&amp;EOMONTH($A44,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A44,0)) + SUMIFS('Chase'!E:E,'Chase'!A:A,"&gt;="&amp;EOMONTH($A44,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A44,0)) + SUMIFS('Wellsfargo'!E:E,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A44,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A44,0)) + SUMIFS('Vyral'!E:E,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A44,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A44,0))</f>
+        <v/>
+      </c>
+      <c r="D44" s="15">
+        <f>SUMIFS('Current'!F:F,'Current'!A:A,"&gt;="&amp;EOMONTH($A44,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A44,0)) + SUMIFS('Chase'!F:F,'Chase'!A:A,"&gt;="&amp;EOMONTH($A44,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A44,0)) + SUMIFS('Wellsfargo'!F:F,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A44,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A44,0)) + SUMIFS('Vyral'!F:F,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A44,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A44,0))</f>
+        <v/>
+      </c>
+      <c r="E44" s="15">
+        <f>B44-C44-D44</f>
+        <v/>
+      </c>
+      <c r="F44" s="9">
+        <f>SUMIFS('Ghana City'!D:D,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A44,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A44,0))</f>
+        <v/>
+      </c>
+      <c r="G44" s="9">
+        <f>SUMIFS('Ghana City'!E:E,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A44,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A44,0))</f>
+        <v/>
+      </c>
+      <c r="H44" s="9">
+        <f>SUMIFS('Ghana City'!F:F,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A44,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A44,0))</f>
+        <v/>
+      </c>
+      <c r="I44" s="9">
+        <f>F44-G44-H44</f>
+        <v/>
+      </c>
+      <c r="J44" s="15">
+        <f>SUMIFS('Credit Card 1'!D:D,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A44,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A44,0)) + SUMIFS('Credit Card 2'!D:D,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A44,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A44,0))</f>
+        <v/>
+      </c>
+      <c r="K44" s="15">
+        <f>SUMIFS('Credit Card 1'!E:E,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A44,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A44,0)) + SUMIFS('Credit Card 2'!E:E,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A44,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A44,0))</f>
+        <v/>
+      </c>
+      <c r="L44" s="15">
+        <f>SUMIFS('Credit Card 1'!F:F,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A44,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A44,0)) + SUMIFS('Credit Card 2'!F:F,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A44,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A44,0))</f>
+        <v/>
+      </c>
+      <c r="M44" s="15">
+        <f>K44+L44-J44</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="19" t="n">
+        <v>46569</v>
+      </c>
+      <c r="B45" s="15">
+        <f>SUMIFS('Current'!D:D,'Current'!A:A,"&gt;="&amp;EOMONTH($A45,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A45,0)) + SUMIFS('Chase'!D:D,'Chase'!A:A,"&gt;="&amp;EOMONTH($A45,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A45,0)) + SUMIFS('Wellsfargo'!D:D,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A45,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A45,0)) + SUMIFS('Vyral'!D:D,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A45,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A45,0))</f>
+        <v/>
+      </c>
+      <c r="C45" s="15">
+        <f>SUMIFS('Current'!E:E,'Current'!A:A,"&gt;="&amp;EOMONTH($A45,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A45,0)) + SUMIFS('Chase'!E:E,'Chase'!A:A,"&gt;="&amp;EOMONTH($A45,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A45,0)) + SUMIFS('Wellsfargo'!E:E,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A45,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A45,0)) + SUMIFS('Vyral'!E:E,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A45,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A45,0))</f>
+        <v/>
+      </c>
+      <c r="D45" s="15">
+        <f>SUMIFS('Current'!F:F,'Current'!A:A,"&gt;="&amp;EOMONTH($A45,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A45,0)) + SUMIFS('Chase'!F:F,'Chase'!A:A,"&gt;="&amp;EOMONTH($A45,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A45,0)) + SUMIFS('Wellsfargo'!F:F,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A45,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A45,0)) + SUMIFS('Vyral'!F:F,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A45,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A45,0))</f>
+        <v/>
+      </c>
+      <c r="E45" s="15">
+        <f>B45-C45-D45</f>
+        <v/>
+      </c>
+      <c r="F45" s="9">
+        <f>SUMIFS('Ghana City'!D:D,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A45,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A45,0))</f>
+        <v/>
+      </c>
+      <c r="G45" s="9">
+        <f>SUMIFS('Ghana City'!E:E,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A45,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A45,0))</f>
+        <v/>
+      </c>
+      <c r="H45" s="9">
+        <f>SUMIFS('Ghana City'!F:F,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A45,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A45,0))</f>
+        <v/>
+      </c>
+      <c r="I45" s="9">
+        <f>F45-G45-H45</f>
+        <v/>
+      </c>
+      <c r="J45" s="15">
+        <f>SUMIFS('Credit Card 1'!D:D,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A45,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A45,0)) + SUMIFS('Credit Card 2'!D:D,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A45,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A45,0))</f>
+        <v/>
+      </c>
+      <c r="K45" s="15">
+        <f>SUMIFS('Credit Card 1'!E:E,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A45,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A45,0)) + SUMIFS('Credit Card 2'!E:E,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A45,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A45,0))</f>
+        <v/>
+      </c>
+      <c r="L45" s="15">
+        <f>SUMIFS('Credit Card 1'!F:F,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A45,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A45,0)) + SUMIFS('Credit Card 2'!F:F,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A45,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A45,0))</f>
+        <v/>
+      </c>
+      <c r="M45" s="15">
+        <f>K45+L45-J45</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="19" t="n">
+        <v>46600</v>
+      </c>
+      <c r="B46" s="15">
+        <f>SUMIFS('Current'!D:D,'Current'!A:A,"&gt;="&amp;EOMONTH($A46,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A46,0)) + SUMIFS('Chase'!D:D,'Chase'!A:A,"&gt;="&amp;EOMONTH($A46,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A46,0)) + SUMIFS('Wellsfargo'!D:D,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A46,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A46,0)) + SUMIFS('Vyral'!D:D,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A46,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A46,0))</f>
+        <v/>
+      </c>
+      <c r="C46" s="15">
+        <f>SUMIFS('Current'!E:E,'Current'!A:A,"&gt;="&amp;EOMONTH($A46,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A46,0)) + SUMIFS('Chase'!E:E,'Chase'!A:A,"&gt;="&amp;EOMONTH($A46,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A46,0)) + SUMIFS('Wellsfargo'!E:E,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A46,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A46,0)) + SUMIFS('Vyral'!E:E,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A46,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A46,0))</f>
+        <v/>
+      </c>
+      <c r="D46" s="15">
+        <f>SUMIFS('Current'!F:F,'Current'!A:A,"&gt;="&amp;EOMONTH($A46,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A46,0)) + SUMIFS('Chase'!F:F,'Chase'!A:A,"&gt;="&amp;EOMONTH($A46,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A46,0)) + SUMIFS('Wellsfargo'!F:F,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A46,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A46,0)) + SUMIFS('Vyral'!F:F,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A46,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A46,0))</f>
+        <v/>
+      </c>
+      <c r="E46" s="15">
+        <f>B46-C46-D46</f>
+        <v/>
+      </c>
+      <c r="F46" s="9">
+        <f>SUMIFS('Ghana City'!D:D,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A46,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A46,0))</f>
+        <v/>
+      </c>
+      <c r="G46" s="9">
+        <f>SUMIFS('Ghana City'!E:E,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A46,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A46,0))</f>
+        <v/>
+      </c>
+      <c r="H46" s="9">
+        <f>SUMIFS('Ghana City'!F:F,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A46,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A46,0))</f>
+        <v/>
+      </c>
+      <c r="I46" s="9">
+        <f>F46-G46-H46</f>
+        <v/>
+      </c>
+      <c r="J46" s="15">
+        <f>SUMIFS('Credit Card 1'!D:D,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A46,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A46,0)) + SUMIFS('Credit Card 2'!D:D,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A46,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A46,0))</f>
+        <v/>
+      </c>
+      <c r="K46" s="15">
+        <f>SUMIFS('Credit Card 1'!E:E,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A46,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A46,0)) + SUMIFS('Credit Card 2'!E:E,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A46,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A46,0))</f>
+        <v/>
+      </c>
+      <c r="L46" s="15">
+        <f>SUMIFS('Credit Card 1'!F:F,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A46,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A46,0)) + SUMIFS('Credit Card 2'!F:F,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A46,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A46,0))</f>
+        <v/>
+      </c>
+      <c r="M46" s="15">
+        <f>K46+L46-J46</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="19" t="n">
+        <v>46631</v>
+      </c>
+      <c r="B47" s="15">
+        <f>SUMIFS('Current'!D:D,'Current'!A:A,"&gt;="&amp;EOMONTH($A47,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A47,0)) + SUMIFS('Chase'!D:D,'Chase'!A:A,"&gt;="&amp;EOMONTH($A47,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A47,0)) + SUMIFS('Wellsfargo'!D:D,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A47,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A47,0)) + SUMIFS('Vyral'!D:D,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A47,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A47,0))</f>
+        <v/>
+      </c>
+      <c r="C47" s="15">
+        <f>SUMIFS('Current'!E:E,'Current'!A:A,"&gt;="&amp;EOMONTH($A47,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A47,0)) + SUMIFS('Chase'!E:E,'Chase'!A:A,"&gt;="&amp;EOMONTH($A47,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A47,0)) + SUMIFS('Wellsfargo'!E:E,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A47,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A47,0)) + SUMIFS('Vyral'!E:E,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A47,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A47,0))</f>
+        <v/>
+      </c>
+      <c r="D47" s="15">
+        <f>SUMIFS('Current'!F:F,'Current'!A:A,"&gt;="&amp;EOMONTH($A47,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A47,0)) + SUMIFS('Chase'!F:F,'Chase'!A:A,"&gt;="&amp;EOMONTH($A47,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A47,0)) + SUMIFS('Wellsfargo'!F:F,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A47,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A47,0)) + SUMIFS('Vyral'!F:F,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A47,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A47,0))</f>
+        <v/>
+      </c>
+      <c r="E47" s="15">
+        <f>B47-C47-D47</f>
+        <v/>
+      </c>
+      <c r="F47" s="9">
+        <f>SUMIFS('Ghana City'!D:D,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A47,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A47,0))</f>
+        <v/>
+      </c>
+      <c r="G47" s="9">
+        <f>SUMIFS('Ghana City'!E:E,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A47,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A47,0))</f>
+        <v/>
+      </c>
+      <c r="H47" s="9">
+        <f>SUMIFS('Ghana City'!F:F,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A47,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A47,0))</f>
+        <v/>
+      </c>
+      <c r="I47" s="9">
+        <f>F47-G47-H47</f>
+        <v/>
+      </c>
+      <c r="J47" s="15">
+        <f>SUMIFS('Credit Card 1'!D:D,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A47,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A47,0)) + SUMIFS('Credit Card 2'!D:D,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A47,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A47,0))</f>
+        <v/>
+      </c>
+      <c r="K47" s="15">
+        <f>SUMIFS('Credit Card 1'!E:E,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A47,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A47,0)) + SUMIFS('Credit Card 2'!E:E,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A47,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A47,0))</f>
+        <v/>
+      </c>
+      <c r="L47" s="15">
+        <f>SUMIFS('Credit Card 1'!F:F,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A47,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A47,0)) + SUMIFS('Credit Card 2'!F:F,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A47,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A47,0))</f>
+        <v/>
+      </c>
+      <c r="M47" s="15">
+        <f>K47+L47-J47</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="19" t="n">
+        <v>46661</v>
+      </c>
+      <c r="B48" s="15">
+        <f>SUMIFS('Current'!D:D,'Current'!A:A,"&gt;="&amp;EOMONTH($A48,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A48,0)) + SUMIFS('Chase'!D:D,'Chase'!A:A,"&gt;="&amp;EOMONTH($A48,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A48,0)) + SUMIFS('Wellsfargo'!D:D,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A48,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A48,0)) + SUMIFS('Vyral'!D:D,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A48,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A48,0))</f>
+        <v/>
+      </c>
+      <c r="C48" s="15">
+        <f>SUMIFS('Current'!E:E,'Current'!A:A,"&gt;="&amp;EOMONTH($A48,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A48,0)) + SUMIFS('Chase'!E:E,'Chase'!A:A,"&gt;="&amp;EOMONTH($A48,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A48,0)) + SUMIFS('Wellsfargo'!E:E,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A48,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A48,0)) + SUMIFS('Vyral'!E:E,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A48,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A48,0))</f>
+        <v/>
+      </c>
+      <c r="D48" s="15">
+        <f>SUMIFS('Current'!F:F,'Current'!A:A,"&gt;="&amp;EOMONTH($A48,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A48,0)) + SUMIFS('Chase'!F:F,'Chase'!A:A,"&gt;="&amp;EOMONTH($A48,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A48,0)) + SUMIFS('Wellsfargo'!F:F,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A48,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A48,0)) + SUMIFS('Vyral'!F:F,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A48,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A48,0))</f>
+        <v/>
+      </c>
+      <c r="E48" s="15">
+        <f>B48-C48-D48</f>
+        <v/>
+      </c>
+      <c r="F48" s="9">
+        <f>SUMIFS('Ghana City'!D:D,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A48,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A48,0))</f>
+        <v/>
+      </c>
+      <c r="G48" s="9">
+        <f>SUMIFS('Ghana City'!E:E,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A48,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A48,0))</f>
+        <v/>
+      </c>
+      <c r="H48" s="9">
+        <f>SUMIFS('Ghana City'!F:F,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A48,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A48,0))</f>
+        <v/>
+      </c>
+      <c r="I48" s="9">
+        <f>F48-G48-H48</f>
+        <v/>
+      </c>
+      <c r="J48" s="15">
+        <f>SUMIFS('Credit Card 1'!D:D,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A48,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A48,0)) + SUMIFS('Credit Card 2'!D:D,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A48,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A48,0))</f>
+        <v/>
+      </c>
+      <c r="K48" s="15">
+        <f>SUMIFS('Credit Card 1'!E:E,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A48,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A48,0)) + SUMIFS('Credit Card 2'!E:E,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A48,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A48,0))</f>
+        <v/>
+      </c>
+      <c r="L48" s="15">
+        <f>SUMIFS('Credit Card 1'!F:F,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A48,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A48,0)) + SUMIFS('Credit Card 2'!F:F,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A48,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A48,0))</f>
+        <v/>
+      </c>
+      <c r="M48" s="15">
+        <f>K48+L48-J48</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="19" t="n">
+        <v>46692</v>
+      </c>
+      <c r="B49" s="15">
+        <f>SUMIFS('Current'!D:D,'Current'!A:A,"&gt;="&amp;EOMONTH($A49,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A49,0)) + SUMIFS('Chase'!D:D,'Chase'!A:A,"&gt;="&amp;EOMONTH($A49,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A49,0)) + SUMIFS('Wellsfargo'!D:D,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A49,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A49,0)) + SUMIFS('Vyral'!D:D,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A49,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A49,0))</f>
+        <v/>
+      </c>
+      <c r="C49" s="15">
+        <f>SUMIFS('Current'!E:E,'Current'!A:A,"&gt;="&amp;EOMONTH($A49,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A49,0)) + SUMIFS('Chase'!E:E,'Chase'!A:A,"&gt;="&amp;EOMONTH($A49,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A49,0)) + SUMIFS('Wellsfargo'!E:E,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A49,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A49,0)) + SUMIFS('Vyral'!E:E,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A49,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A49,0))</f>
+        <v/>
+      </c>
+      <c r="D49" s="15">
+        <f>SUMIFS('Current'!F:F,'Current'!A:A,"&gt;="&amp;EOMONTH($A49,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A49,0)) + SUMIFS('Chase'!F:F,'Chase'!A:A,"&gt;="&amp;EOMONTH($A49,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A49,0)) + SUMIFS('Wellsfargo'!F:F,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A49,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A49,0)) + SUMIFS('Vyral'!F:F,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A49,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A49,0))</f>
+        <v/>
+      </c>
+      <c r="E49" s="15">
+        <f>B49-C49-D49</f>
+        <v/>
+      </c>
+      <c r="F49" s="9">
+        <f>SUMIFS('Ghana City'!D:D,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A49,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A49,0))</f>
+        <v/>
+      </c>
+      <c r="G49" s="9">
+        <f>SUMIFS('Ghana City'!E:E,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A49,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A49,0))</f>
+        <v/>
+      </c>
+      <c r="H49" s="9">
+        <f>SUMIFS('Ghana City'!F:F,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A49,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A49,0))</f>
+        <v/>
+      </c>
+      <c r="I49" s="9">
+        <f>F49-G49-H49</f>
+        <v/>
+      </c>
+      <c r="J49" s="15">
+        <f>SUMIFS('Credit Card 1'!D:D,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A49,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A49,0)) + SUMIFS('Credit Card 2'!D:D,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A49,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A49,0))</f>
+        <v/>
+      </c>
+      <c r="K49" s="15">
+        <f>SUMIFS('Credit Card 1'!E:E,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A49,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A49,0)) + SUMIFS('Credit Card 2'!E:E,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A49,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A49,0))</f>
+        <v/>
+      </c>
+      <c r="L49" s="15">
+        <f>SUMIFS('Credit Card 1'!F:F,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A49,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A49,0)) + SUMIFS('Credit Card 2'!F:F,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A49,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A49,0))</f>
+        <v/>
+      </c>
+      <c r="M49" s="15">
+        <f>K49+L49-J49</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="19" t="n">
+        <v>46722</v>
+      </c>
+      <c r="B50" s="15">
+        <f>SUMIFS('Current'!D:D,'Current'!A:A,"&gt;="&amp;EOMONTH($A50,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A50,0)) + SUMIFS('Chase'!D:D,'Chase'!A:A,"&gt;="&amp;EOMONTH($A50,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A50,0)) + SUMIFS('Wellsfargo'!D:D,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A50,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A50,0)) + SUMIFS('Vyral'!D:D,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A50,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A50,0))</f>
+        <v/>
+      </c>
+      <c r="C50" s="15">
+        <f>SUMIFS('Current'!E:E,'Current'!A:A,"&gt;="&amp;EOMONTH($A50,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A50,0)) + SUMIFS('Chase'!E:E,'Chase'!A:A,"&gt;="&amp;EOMONTH($A50,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A50,0)) + SUMIFS('Wellsfargo'!E:E,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A50,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A50,0)) + SUMIFS('Vyral'!E:E,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A50,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A50,0))</f>
+        <v/>
+      </c>
+      <c r="D50" s="15">
+        <f>SUMIFS('Current'!F:F,'Current'!A:A,"&gt;="&amp;EOMONTH($A50,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A50,0)) + SUMIFS('Chase'!F:F,'Chase'!A:A,"&gt;="&amp;EOMONTH($A50,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A50,0)) + SUMIFS('Wellsfargo'!F:F,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A50,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A50,0)) + SUMIFS('Vyral'!F:F,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A50,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A50,0))</f>
+        <v/>
+      </c>
+      <c r="E50" s="15">
+        <f>B50-C50-D50</f>
+        <v/>
+      </c>
+      <c r="F50" s="9">
+        <f>SUMIFS('Ghana City'!D:D,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A50,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A50,0))</f>
+        <v/>
+      </c>
+      <c r="G50" s="9">
+        <f>SUMIFS('Ghana City'!E:E,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A50,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A50,0))</f>
+        <v/>
+      </c>
+      <c r="H50" s="9">
+        <f>SUMIFS('Ghana City'!F:F,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A50,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A50,0))</f>
+        <v/>
+      </c>
+      <c r="I50" s="9">
+        <f>F50-G50-H50</f>
+        <v/>
+      </c>
+      <c r="J50" s="15">
+        <f>SUMIFS('Credit Card 1'!D:D,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A50,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A50,0)) + SUMIFS('Credit Card 2'!D:D,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A50,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A50,0))</f>
+        <v/>
+      </c>
+      <c r="K50" s="15">
+        <f>SUMIFS('Credit Card 1'!E:E,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A50,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A50,0)) + SUMIFS('Credit Card 2'!E:E,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A50,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A50,0))</f>
+        <v/>
+      </c>
+      <c r="L50" s="15">
+        <f>SUMIFS('Credit Card 1'!F:F,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A50,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A50,0)) + SUMIFS('Credit Card 2'!F:F,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A50,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A50,0))</f>
+        <v/>
+      </c>
+      <c r="M50" s="15">
+        <f>K50+L50-J50</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="19" t="n">
+        <v>46753</v>
+      </c>
+      <c r="B51" s="15">
+        <f>SUMIFS('Current'!D:D,'Current'!A:A,"&gt;="&amp;EOMONTH($A51,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A51,0)) + SUMIFS('Chase'!D:D,'Chase'!A:A,"&gt;="&amp;EOMONTH($A51,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A51,0)) + SUMIFS('Wellsfargo'!D:D,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A51,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A51,0)) + SUMIFS('Vyral'!D:D,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A51,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A51,0))</f>
+        <v/>
+      </c>
+      <c r="C51" s="15">
+        <f>SUMIFS('Current'!E:E,'Current'!A:A,"&gt;="&amp;EOMONTH($A51,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A51,0)) + SUMIFS('Chase'!E:E,'Chase'!A:A,"&gt;="&amp;EOMONTH($A51,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A51,0)) + SUMIFS('Wellsfargo'!E:E,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A51,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A51,0)) + SUMIFS('Vyral'!E:E,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A51,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A51,0))</f>
+        <v/>
+      </c>
+      <c r="D51" s="15">
+        <f>SUMIFS('Current'!F:F,'Current'!A:A,"&gt;="&amp;EOMONTH($A51,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A51,0)) + SUMIFS('Chase'!F:F,'Chase'!A:A,"&gt;="&amp;EOMONTH($A51,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A51,0)) + SUMIFS('Wellsfargo'!F:F,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A51,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A51,0)) + SUMIFS('Vyral'!F:F,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A51,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A51,0))</f>
+        <v/>
+      </c>
+      <c r="E51" s="15">
+        <f>B51-C51-D51</f>
+        <v/>
+      </c>
+      <c r="F51" s="9">
+        <f>SUMIFS('Ghana City'!D:D,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A51,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A51,0))</f>
+        <v/>
+      </c>
+      <c r="G51" s="9">
+        <f>SUMIFS('Ghana City'!E:E,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A51,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A51,0))</f>
+        <v/>
+      </c>
+      <c r="H51" s="9">
+        <f>SUMIFS('Ghana City'!F:F,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A51,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A51,0))</f>
+        <v/>
+      </c>
+      <c r="I51" s="9">
+        <f>F51-G51-H51</f>
+        <v/>
+      </c>
+      <c r="J51" s="15">
+        <f>SUMIFS('Credit Card 1'!D:D,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A51,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A51,0)) + SUMIFS('Credit Card 2'!D:D,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A51,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A51,0))</f>
+        <v/>
+      </c>
+      <c r="K51" s="15">
+        <f>SUMIFS('Credit Card 1'!E:E,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A51,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A51,0)) + SUMIFS('Credit Card 2'!E:E,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A51,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A51,0))</f>
+        <v/>
+      </c>
+      <c r="L51" s="15">
+        <f>SUMIFS('Credit Card 1'!F:F,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A51,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A51,0)) + SUMIFS('Credit Card 2'!F:F,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A51,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A51,0))</f>
+        <v/>
+      </c>
+      <c r="M51" s="15">
+        <f>K51+L51-J51</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="19" t="n">
+        <v>46784</v>
+      </c>
+      <c r="B52" s="15">
+        <f>SUMIFS('Current'!D:D,'Current'!A:A,"&gt;="&amp;EOMONTH($A52,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A52,0)) + SUMIFS('Chase'!D:D,'Chase'!A:A,"&gt;="&amp;EOMONTH($A52,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A52,0)) + SUMIFS('Wellsfargo'!D:D,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A52,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A52,0)) + SUMIFS('Vyral'!D:D,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A52,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A52,0))</f>
+        <v/>
+      </c>
+      <c r="C52" s="15">
+        <f>SUMIFS('Current'!E:E,'Current'!A:A,"&gt;="&amp;EOMONTH($A52,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A52,0)) + SUMIFS('Chase'!E:E,'Chase'!A:A,"&gt;="&amp;EOMONTH($A52,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A52,0)) + SUMIFS('Wellsfargo'!E:E,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A52,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A52,0)) + SUMIFS('Vyral'!E:E,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A52,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A52,0))</f>
+        <v/>
+      </c>
+      <c r="D52" s="15">
+        <f>SUMIFS('Current'!F:F,'Current'!A:A,"&gt;="&amp;EOMONTH($A52,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A52,0)) + SUMIFS('Chase'!F:F,'Chase'!A:A,"&gt;="&amp;EOMONTH($A52,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A52,0)) + SUMIFS('Wellsfargo'!F:F,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A52,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A52,0)) + SUMIFS('Vyral'!F:F,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A52,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A52,0))</f>
+        <v/>
+      </c>
+      <c r="E52" s="15">
+        <f>B52-C52-D52</f>
+        <v/>
+      </c>
+      <c r="F52" s="9">
+        <f>SUMIFS('Ghana City'!D:D,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A52,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A52,0))</f>
+        <v/>
+      </c>
+      <c r="G52" s="9">
+        <f>SUMIFS('Ghana City'!E:E,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A52,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A52,0))</f>
+        <v/>
+      </c>
+      <c r="H52" s="9">
+        <f>SUMIFS('Ghana City'!F:F,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A52,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A52,0))</f>
+        <v/>
+      </c>
+      <c r="I52" s="9">
+        <f>F52-G52-H52</f>
+        <v/>
+      </c>
+      <c r="J52" s="15">
+        <f>SUMIFS('Credit Card 1'!D:D,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A52,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A52,0)) + SUMIFS('Credit Card 2'!D:D,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A52,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A52,0))</f>
+        <v/>
+      </c>
+      <c r="K52" s="15">
+        <f>SUMIFS('Credit Card 1'!E:E,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A52,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A52,0)) + SUMIFS('Credit Card 2'!E:E,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A52,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A52,0))</f>
+        <v/>
+      </c>
+      <c r="L52" s="15">
+        <f>SUMIFS('Credit Card 1'!F:F,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A52,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A52,0)) + SUMIFS('Credit Card 2'!F:F,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A52,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A52,0))</f>
+        <v/>
+      </c>
+      <c r="M52" s="15">
+        <f>K52+L52-J52</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="19" t="n">
+        <v>46813</v>
+      </c>
+      <c r="B53" s="15">
+        <f>SUMIFS('Current'!D:D,'Current'!A:A,"&gt;="&amp;EOMONTH($A53,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A53,0)) + SUMIFS('Chase'!D:D,'Chase'!A:A,"&gt;="&amp;EOMONTH($A53,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A53,0)) + SUMIFS('Wellsfargo'!D:D,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A53,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A53,0)) + SUMIFS('Vyral'!D:D,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A53,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A53,0))</f>
+        <v/>
+      </c>
+      <c r="C53" s="15">
+        <f>SUMIFS('Current'!E:E,'Current'!A:A,"&gt;="&amp;EOMONTH($A53,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A53,0)) + SUMIFS('Chase'!E:E,'Chase'!A:A,"&gt;="&amp;EOMONTH($A53,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A53,0)) + SUMIFS('Wellsfargo'!E:E,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A53,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A53,0)) + SUMIFS('Vyral'!E:E,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A53,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A53,0))</f>
+        <v/>
+      </c>
+      <c r="D53" s="15">
+        <f>SUMIFS('Current'!F:F,'Current'!A:A,"&gt;="&amp;EOMONTH($A53,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A53,0)) + SUMIFS('Chase'!F:F,'Chase'!A:A,"&gt;="&amp;EOMONTH($A53,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A53,0)) + SUMIFS('Wellsfargo'!F:F,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A53,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A53,0)) + SUMIFS('Vyral'!F:F,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A53,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A53,0))</f>
+        <v/>
+      </c>
+      <c r="E53" s="15">
+        <f>B53-C53-D53</f>
+        <v/>
+      </c>
+      <c r="F53" s="9">
+        <f>SUMIFS('Ghana City'!D:D,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A53,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A53,0))</f>
+        <v/>
+      </c>
+      <c r="G53" s="9">
+        <f>SUMIFS('Ghana City'!E:E,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A53,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A53,0))</f>
+        <v/>
+      </c>
+      <c r="H53" s="9">
+        <f>SUMIFS('Ghana City'!F:F,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A53,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A53,0))</f>
+        <v/>
+      </c>
+      <c r="I53" s="9">
+        <f>F53-G53-H53</f>
+        <v/>
+      </c>
+      <c r="J53" s="15">
+        <f>SUMIFS('Credit Card 1'!D:D,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A53,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A53,0)) + SUMIFS('Credit Card 2'!D:D,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A53,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A53,0))</f>
+        <v/>
+      </c>
+      <c r="K53" s="15">
+        <f>SUMIFS('Credit Card 1'!E:E,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A53,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A53,0)) + SUMIFS('Credit Card 2'!E:E,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A53,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A53,0))</f>
+        <v/>
+      </c>
+      <c r="L53" s="15">
+        <f>SUMIFS('Credit Card 1'!F:F,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A53,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A53,0)) + SUMIFS('Credit Card 2'!F:F,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A53,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A53,0))</f>
+        <v/>
+      </c>
+      <c r="M53" s="15">
+        <f>K53+L53-J53</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="19" t="n">
+        <v>46844</v>
+      </c>
+      <c r="B54" s="15">
+        <f>SUMIFS('Current'!D:D,'Current'!A:A,"&gt;="&amp;EOMONTH($A54,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A54,0)) + SUMIFS('Chase'!D:D,'Chase'!A:A,"&gt;="&amp;EOMONTH($A54,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A54,0)) + SUMIFS('Wellsfargo'!D:D,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A54,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A54,0)) + SUMIFS('Vyral'!D:D,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A54,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A54,0))</f>
+        <v/>
+      </c>
+      <c r="C54" s="15">
+        <f>SUMIFS('Current'!E:E,'Current'!A:A,"&gt;="&amp;EOMONTH($A54,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A54,0)) + SUMIFS('Chase'!E:E,'Chase'!A:A,"&gt;="&amp;EOMONTH($A54,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A54,0)) + SUMIFS('Wellsfargo'!E:E,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A54,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A54,0)) + SUMIFS('Vyral'!E:E,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A54,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A54,0))</f>
+        <v/>
+      </c>
+      <c r="D54" s="15">
+        <f>SUMIFS('Current'!F:F,'Current'!A:A,"&gt;="&amp;EOMONTH($A54,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A54,0)) + SUMIFS('Chase'!F:F,'Chase'!A:A,"&gt;="&amp;EOMONTH($A54,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A54,0)) + SUMIFS('Wellsfargo'!F:F,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A54,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A54,0)) + SUMIFS('Vyral'!F:F,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A54,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A54,0))</f>
+        <v/>
+      </c>
+      <c r="E54" s="15">
+        <f>B54-C54-D54</f>
+        <v/>
+      </c>
+      <c r="F54" s="9">
+        <f>SUMIFS('Ghana City'!D:D,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A54,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A54,0))</f>
+        <v/>
+      </c>
+      <c r="G54" s="9">
+        <f>SUMIFS('Ghana City'!E:E,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A54,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A54,0))</f>
+        <v/>
+      </c>
+      <c r="H54" s="9">
+        <f>SUMIFS('Ghana City'!F:F,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A54,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A54,0))</f>
+        <v/>
+      </c>
+      <c r="I54" s="9">
+        <f>F54-G54-H54</f>
+        <v/>
+      </c>
+      <c r="J54" s="15">
+        <f>SUMIFS('Credit Card 1'!D:D,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A54,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A54,0)) + SUMIFS('Credit Card 2'!D:D,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A54,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A54,0))</f>
+        <v/>
+      </c>
+      <c r="K54" s="15">
+        <f>SUMIFS('Credit Card 1'!E:E,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A54,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A54,0)) + SUMIFS('Credit Card 2'!E:E,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A54,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A54,0))</f>
+        <v/>
+      </c>
+      <c r="L54" s="15">
+        <f>SUMIFS('Credit Card 1'!F:F,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A54,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A54,0)) + SUMIFS('Credit Card 2'!F:F,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A54,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A54,0))</f>
+        <v/>
+      </c>
+      <c r="M54" s="15">
+        <f>K54+L54-J54</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="19" t="n">
+        <v>46874</v>
+      </c>
+      <c r="B55" s="15">
+        <f>SUMIFS('Current'!D:D,'Current'!A:A,"&gt;="&amp;EOMONTH($A55,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A55,0)) + SUMIFS('Chase'!D:D,'Chase'!A:A,"&gt;="&amp;EOMONTH($A55,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A55,0)) + SUMIFS('Wellsfargo'!D:D,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A55,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A55,0)) + SUMIFS('Vyral'!D:D,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A55,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A55,0))</f>
+        <v/>
+      </c>
+      <c r="C55" s="15">
+        <f>SUMIFS('Current'!E:E,'Current'!A:A,"&gt;="&amp;EOMONTH($A55,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A55,0)) + SUMIFS('Chase'!E:E,'Chase'!A:A,"&gt;="&amp;EOMONTH($A55,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A55,0)) + SUMIFS('Wellsfargo'!E:E,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A55,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A55,0)) + SUMIFS('Vyral'!E:E,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A55,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A55,0))</f>
+        <v/>
+      </c>
+      <c r="D55" s="15">
+        <f>SUMIFS('Current'!F:F,'Current'!A:A,"&gt;="&amp;EOMONTH($A55,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A55,0)) + SUMIFS('Chase'!F:F,'Chase'!A:A,"&gt;="&amp;EOMONTH($A55,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A55,0)) + SUMIFS('Wellsfargo'!F:F,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A55,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A55,0)) + SUMIFS('Vyral'!F:F,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A55,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A55,0))</f>
+        <v/>
+      </c>
+      <c r="E55" s="15">
+        <f>B55-C55-D55</f>
+        <v/>
+      </c>
+      <c r="F55" s="9">
+        <f>SUMIFS('Ghana City'!D:D,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A55,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A55,0))</f>
+        <v/>
+      </c>
+      <c r="G55" s="9">
+        <f>SUMIFS('Ghana City'!E:E,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A55,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A55,0))</f>
+        <v/>
+      </c>
+      <c r="H55" s="9">
+        <f>SUMIFS('Ghana City'!F:F,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A55,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A55,0))</f>
+        <v/>
+      </c>
+      <c r="I55" s="9">
+        <f>F55-G55-H55</f>
+        <v/>
+      </c>
+      <c r="J55" s="15">
+        <f>SUMIFS('Credit Card 1'!D:D,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A55,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A55,0)) + SUMIFS('Credit Card 2'!D:D,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A55,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A55,0))</f>
+        <v/>
+      </c>
+      <c r="K55" s="15">
+        <f>SUMIFS('Credit Card 1'!E:E,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A55,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A55,0)) + SUMIFS('Credit Card 2'!E:E,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A55,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A55,0))</f>
+        <v/>
+      </c>
+      <c r="L55" s="15">
+        <f>SUMIFS('Credit Card 1'!F:F,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A55,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A55,0)) + SUMIFS('Credit Card 2'!F:F,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A55,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A55,0))</f>
+        <v/>
+      </c>
+      <c r="M55" s="15">
+        <f>K55+L55-J55</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="19" t="n">
+        <v>46905</v>
+      </c>
+      <c r="B56" s="15">
+        <f>SUMIFS('Current'!D:D,'Current'!A:A,"&gt;="&amp;EOMONTH($A56,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A56,0)) + SUMIFS('Chase'!D:D,'Chase'!A:A,"&gt;="&amp;EOMONTH($A56,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A56,0)) + SUMIFS('Wellsfargo'!D:D,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A56,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A56,0)) + SUMIFS('Vyral'!D:D,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A56,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A56,0))</f>
+        <v/>
+      </c>
+      <c r="C56" s="15">
+        <f>SUMIFS('Current'!E:E,'Current'!A:A,"&gt;="&amp;EOMONTH($A56,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A56,0)) + SUMIFS('Chase'!E:E,'Chase'!A:A,"&gt;="&amp;EOMONTH($A56,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A56,0)) + SUMIFS('Wellsfargo'!E:E,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A56,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A56,0)) + SUMIFS('Vyral'!E:E,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A56,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A56,0))</f>
+        <v/>
+      </c>
+      <c r="D56" s="15">
+        <f>SUMIFS('Current'!F:F,'Current'!A:A,"&gt;="&amp;EOMONTH($A56,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A56,0)) + SUMIFS('Chase'!F:F,'Chase'!A:A,"&gt;="&amp;EOMONTH($A56,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A56,0)) + SUMIFS('Wellsfargo'!F:F,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A56,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A56,0)) + SUMIFS('Vyral'!F:F,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A56,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A56,0))</f>
+        <v/>
+      </c>
+      <c r="E56" s="15">
+        <f>B56-C56-D56</f>
+        <v/>
+      </c>
+      <c r="F56" s="9">
+        <f>SUMIFS('Ghana City'!D:D,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A56,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A56,0))</f>
+        <v/>
+      </c>
+      <c r="G56" s="9">
+        <f>SUMIFS('Ghana City'!E:E,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A56,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A56,0))</f>
+        <v/>
+      </c>
+      <c r="H56" s="9">
+        <f>SUMIFS('Ghana City'!F:F,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A56,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A56,0))</f>
+        <v/>
+      </c>
+      <c r="I56" s="9">
+        <f>F56-G56-H56</f>
+        <v/>
+      </c>
+      <c r="J56" s="15">
+        <f>SUMIFS('Credit Card 1'!D:D,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A56,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A56,0)) + SUMIFS('Credit Card 2'!D:D,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A56,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A56,0))</f>
+        <v/>
+      </c>
+      <c r="K56" s="15">
+        <f>SUMIFS('Credit Card 1'!E:E,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A56,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A56,0)) + SUMIFS('Credit Card 2'!E:E,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A56,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A56,0))</f>
+        <v/>
+      </c>
+      <c r="L56" s="15">
+        <f>SUMIFS('Credit Card 1'!F:F,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A56,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A56,0)) + SUMIFS('Credit Card 2'!F:F,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A56,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A56,0))</f>
+        <v/>
+      </c>
+      <c r="M56" s="15">
+        <f>K56+L56-J56</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="19" t="n">
+        <v>46935</v>
+      </c>
+      <c r="B57" s="15">
+        <f>SUMIFS('Current'!D:D,'Current'!A:A,"&gt;="&amp;EOMONTH($A57,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A57,0)) + SUMIFS('Chase'!D:D,'Chase'!A:A,"&gt;="&amp;EOMONTH($A57,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A57,0)) + SUMIFS('Wellsfargo'!D:D,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A57,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A57,0)) + SUMIFS('Vyral'!D:D,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A57,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A57,0))</f>
+        <v/>
+      </c>
+      <c r="C57" s="15">
+        <f>SUMIFS('Current'!E:E,'Current'!A:A,"&gt;="&amp;EOMONTH($A57,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A57,0)) + SUMIFS('Chase'!E:E,'Chase'!A:A,"&gt;="&amp;EOMONTH($A57,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A57,0)) + SUMIFS('Wellsfargo'!E:E,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A57,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A57,0)) + SUMIFS('Vyral'!E:E,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A57,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A57,0))</f>
+        <v/>
+      </c>
+      <c r="D57" s="15">
+        <f>SUMIFS('Current'!F:F,'Current'!A:A,"&gt;="&amp;EOMONTH($A57,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A57,0)) + SUMIFS('Chase'!F:F,'Chase'!A:A,"&gt;="&amp;EOMONTH($A57,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A57,0)) + SUMIFS('Wellsfargo'!F:F,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A57,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A57,0)) + SUMIFS('Vyral'!F:F,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A57,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A57,0))</f>
+        <v/>
+      </c>
+      <c r="E57" s="15">
+        <f>B57-C57-D57</f>
+        <v/>
+      </c>
+      <c r="F57" s="9">
+        <f>SUMIFS('Ghana City'!D:D,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A57,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A57,0))</f>
+        <v/>
+      </c>
+      <c r="G57" s="9">
+        <f>SUMIFS('Ghana City'!E:E,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A57,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A57,0))</f>
+        <v/>
+      </c>
+      <c r="H57" s="9">
+        <f>SUMIFS('Ghana City'!F:F,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A57,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A57,0))</f>
+        <v/>
+      </c>
+      <c r="I57" s="9">
+        <f>F57-G57-H57</f>
+        <v/>
+      </c>
+      <c r="J57" s="15">
+        <f>SUMIFS('Credit Card 1'!D:D,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A57,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A57,0)) + SUMIFS('Credit Card 2'!D:D,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A57,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A57,0))</f>
+        <v/>
+      </c>
+      <c r="K57" s="15">
+        <f>SUMIFS('Credit Card 1'!E:E,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A57,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A57,0)) + SUMIFS('Credit Card 2'!E:E,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A57,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A57,0))</f>
+        <v/>
+      </c>
+      <c r="L57" s="15">
+        <f>SUMIFS('Credit Card 1'!F:F,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A57,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A57,0)) + SUMIFS('Credit Card 2'!F:F,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A57,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A57,0))</f>
+        <v/>
+      </c>
+      <c r="M57" s="15">
+        <f>K57+L57-J57</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="19" t="n">
+        <v>46966</v>
+      </c>
+      <c r="B58" s="15">
+        <f>SUMIFS('Current'!D:D,'Current'!A:A,"&gt;="&amp;EOMONTH($A58,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A58,0)) + SUMIFS('Chase'!D:D,'Chase'!A:A,"&gt;="&amp;EOMONTH($A58,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A58,0)) + SUMIFS('Wellsfargo'!D:D,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A58,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A58,0)) + SUMIFS('Vyral'!D:D,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A58,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A58,0))</f>
+        <v/>
+      </c>
+      <c r="C58" s="15">
+        <f>SUMIFS('Current'!E:E,'Current'!A:A,"&gt;="&amp;EOMONTH($A58,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A58,0)) + SUMIFS('Chase'!E:E,'Chase'!A:A,"&gt;="&amp;EOMONTH($A58,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A58,0)) + SUMIFS('Wellsfargo'!E:E,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A58,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A58,0)) + SUMIFS('Vyral'!E:E,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A58,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A58,0))</f>
+        <v/>
+      </c>
+      <c r="D58" s="15">
+        <f>SUMIFS('Current'!F:F,'Current'!A:A,"&gt;="&amp;EOMONTH($A58,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A58,0)) + SUMIFS('Chase'!F:F,'Chase'!A:A,"&gt;="&amp;EOMONTH($A58,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A58,0)) + SUMIFS('Wellsfargo'!F:F,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A58,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A58,0)) + SUMIFS('Vyral'!F:F,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A58,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A58,0))</f>
+        <v/>
+      </c>
+      <c r="E58" s="15">
+        <f>B58-C58-D58</f>
+        <v/>
+      </c>
+      <c r="F58" s="9">
+        <f>SUMIFS('Ghana City'!D:D,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A58,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A58,0))</f>
+        <v/>
+      </c>
+      <c r="G58" s="9">
+        <f>SUMIFS('Ghana City'!E:E,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A58,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A58,0))</f>
+        <v/>
+      </c>
+      <c r="H58" s="9">
+        <f>SUMIFS('Ghana City'!F:F,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A58,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A58,0))</f>
+        <v/>
+      </c>
+      <c r="I58" s="9">
+        <f>F58-G58-H58</f>
+        <v/>
+      </c>
+      <c r="J58" s="15">
+        <f>SUMIFS('Credit Card 1'!D:D,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A58,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A58,0)) + SUMIFS('Credit Card 2'!D:D,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A58,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A58,0))</f>
+        <v/>
+      </c>
+      <c r="K58" s="15">
+        <f>SUMIFS('Credit Card 1'!E:E,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A58,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A58,0)) + SUMIFS('Credit Card 2'!E:E,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A58,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A58,0))</f>
+        <v/>
+      </c>
+      <c r="L58" s="15">
+        <f>SUMIFS('Credit Card 1'!F:F,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A58,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A58,0)) + SUMIFS('Credit Card 2'!F:F,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A58,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A58,0))</f>
+        <v/>
+      </c>
+      <c r="M58" s="15">
+        <f>K58+L58-J58</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="19" t="n">
+        <v>46997</v>
+      </c>
+      <c r="B59" s="15">
+        <f>SUMIFS('Current'!D:D,'Current'!A:A,"&gt;="&amp;EOMONTH($A59,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A59,0)) + SUMIFS('Chase'!D:D,'Chase'!A:A,"&gt;="&amp;EOMONTH($A59,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A59,0)) + SUMIFS('Wellsfargo'!D:D,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A59,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A59,0)) + SUMIFS('Vyral'!D:D,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A59,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A59,0))</f>
+        <v/>
+      </c>
+      <c r="C59" s="15">
+        <f>SUMIFS('Current'!E:E,'Current'!A:A,"&gt;="&amp;EOMONTH($A59,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A59,0)) + SUMIFS('Chase'!E:E,'Chase'!A:A,"&gt;="&amp;EOMONTH($A59,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A59,0)) + SUMIFS('Wellsfargo'!E:E,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A59,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A59,0)) + SUMIFS('Vyral'!E:E,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A59,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A59,0))</f>
+        <v/>
+      </c>
+      <c r="D59" s="15">
+        <f>SUMIFS('Current'!F:F,'Current'!A:A,"&gt;="&amp;EOMONTH($A59,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A59,0)) + SUMIFS('Chase'!F:F,'Chase'!A:A,"&gt;="&amp;EOMONTH($A59,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A59,0)) + SUMIFS('Wellsfargo'!F:F,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A59,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A59,0)) + SUMIFS('Vyral'!F:F,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A59,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A59,0))</f>
+        <v/>
+      </c>
+      <c r="E59" s="15">
+        <f>B59-C59-D59</f>
+        <v/>
+      </c>
+      <c r="F59" s="9">
+        <f>SUMIFS('Ghana City'!D:D,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A59,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A59,0))</f>
+        <v/>
+      </c>
+      <c r="G59" s="9">
+        <f>SUMIFS('Ghana City'!E:E,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A59,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A59,0))</f>
+        <v/>
+      </c>
+      <c r="H59" s="9">
+        <f>SUMIFS('Ghana City'!F:F,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A59,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A59,0))</f>
+        <v/>
+      </c>
+      <c r="I59" s="9">
+        <f>F59-G59-H59</f>
+        <v/>
+      </c>
+      <c r="J59" s="15">
+        <f>SUMIFS('Credit Card 1'!D:D,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A59,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A59,0)) + SUMIFS('Credit Card 2'!D:D,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A59,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A59,0))</f>
+        <v/>
+      </c>
+      <c r="K59" s="15">
+        <f>SUMIFS('Credit Card 1'!E:E,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A59,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A59,0)) + SUMIFS('Credit Card 2'!E:E,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A59,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A59,0))</f>
+        <v/>
+      </c>
+      <c r="L59" s="15">
+        <f>SUMIFS('Credit Card 1'!F:F,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A59,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A59,0)) + SUMIFS('Credit Card 2'!F:F,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A59,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A59,0))</f>
+        <v/>
+      </c>
+      <c r="M59" s="15">
+        <f>K59+L59-J59</f>
+        <v/>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="19" t="n">
+        <v>47027</v>
+      </c>
+      <c r="B60" s="15">
+        <f>SUMIFS('Current'!D:D,'Current'!A:A,"&gt;="&amp;EOMONTH($A60,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A60,0)) + SUMIFS('Chase'!D:D,'Chase'!A:A,"&gt;="&amp;EOMONTH($A60,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A60,0)) + SUMIFS('Wellsfargo'!D:D,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A60,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A60,0)) + SUMIFS('Vyral'!D:D,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A60,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A60,0))</f>
+        <v/>
+      </c>
+      <c r="C60" s="15">
+        <f>SUMIFS('Current'!E:E,'Current'!A:A,"&gt;="&amp;EOMONTH($A60,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A60,0)) + SUMIFS('Chase'!E:E,'Chase'!A:A,"&gt;="&amp;EOMONTH($A60,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A60,0)) + SUMIFS('Wellsfargo'!E:E,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A60,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A60,0)) + SUMIFS('Vyral'!E:E,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A60,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A60,0))</f>
+        <v/>
+      </c>
+      <c r="D60" s="15">
+        <f>SUMIFS('Current'!F:F,'Current'!A:A,"&gt;="&amp;EOMONTH($A60,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A60,0)) + SUMIFS('Chase'!F:F,'Chase'!A:A,"&gt;="&amp;EOMONTH($A60,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A60,0)) + SUMIFS('Wellsfargo'!F:F,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A60,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A60,0)) + SUMIFS('Vyral'!F:F,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A60,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A60,0))</f>
+        <v/>
+      </c>
+      <c r="E60" s="15">
+        <f>B60-C60-D60</f>
+        <v/>
+      </c>
+      <c r="F60" s="9">
+        <f>SUMIFS('Ghana City'!D:D,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A60,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A60,0))</f>
+        <v/>
+      </c>
+      <c r="G60" s="9">
+        <f>SUMIFS('Ghana City'!E:E,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A60,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A60,0))</f>
+        <v/>
+      </c>
+      <c r="H60" s="9">
+        <f>SUMIFS('Ghana City'!F:F,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A60,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A60,0))</f>
+        <v/>
+      </c>
+      <c r="I60" s="9">
+        <f>F60-G60-H60</f>
+        <v/>
+      </c>
+      <c r="J60" s="15">
+        <f>SUMIFS('Credit Card 1'!D:D,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A60,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A60,0)) + SUMIFS('Credit Card 2'!D:D,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A60,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A60,0))</f>
+        <v/>
+      </c>
+      <c r="K60" s="15">
+        <f>SUMIFS('Credit Card 1'!E:E,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A60,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A60,0)) + SUMIFS('Credit Card 2'!E:E,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A60,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A60,0))</f>
+        <v/>
+      </c>
+      <c r="L60" s="15">
+        <f>SUMIFS('Credit Card 1'!F:F,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A60,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A60,0)) + SUMIFS('Credit Card 2'!F:F,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A60,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A60,0))</f>
+        <v/>
+      </c>
+      <c r="M60" s="15">
+        <f>K60+L60-J60</f>
+        <v/>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="19" t="n">
+        <v>47058</v>
+      </c>
+      <c r="B61" s="15">
+        <f>SUMIFS('Current'!D:D,'Current'!A:A,"&gt;="&amp;EOMONTH($A61,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A61,0)) + SUMIFS('Chase'!D:D,'Chase'!A:A,"&gt;="&amp;EOMONTH($A61,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A61,0)) + SUMIFS('Wellsfargo'!D:D,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A61,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A61,0)) + SUMIFS('Vyral'!D:D,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A61,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A61,0))</f>
+        <v/>
+      </c>
+      <c r="C61" s="15">
+        <f>SUMIFS('Current'!E:E,'Current'!A:A,"&gt;="&amp;EOMONTH($A61,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A61,0)) + SUMIFS('Chase'!E:E,'Chase'!A:A,"&gt;="&amp;EOMONTH($A61,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A61,0)) + SUMIFS('Wellsfargo'!E:E,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A61,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A61,0)) + SUMIFS('Vyral'!E:E,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A61,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A61,0))</f>
+        <v/>
+      </c>
+      <c r="D61" s="15">
+        <f>SUMIFS('Current'!F:F,'Current'!A:A,"&gt;="&amp;EOMONTH($A61,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A61,0)) + SUMIFS('Chase'!F:F,'Chase'!A:A,"&gt;="&amp;EOMONTH($A61,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A61,0)) + SUMIFS('Wellsfargo'!F:F,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A61,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A61,0)) + SUMIFS('Vyral'!F:F,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A61,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A61,0))</f>
+        <v/>
+      </c>
+      <c r="E61" s="15">
+        <f>B61-C61-D61</f>
+        <v/>
+      </c>
+      <c r="F61" s="9">
+        <f>SUMIFS('Ghana City'!D:D,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A61,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A61,0))</f>
+        <v/>
+      </c>
+      <c r="G61" s="9">
+        <f>SUMIFS('Ghana City'!E:E,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A61,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A61,0))</f>
+        <v/>
+      </c>
+      <c r="H61" s="9">
+        <f>SUMIFS('Ghana City'!F:F,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A61,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A61,0))</f>
+        <v/>
+      </c>
+      <c r="I61" s="9">
+        <f>F61-G61-H61</f>
+        <v/>
+      </c>
+      <c r="J61" s="15">
+        <f>SUMIFS('Credit Card 1'!D:D,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A61,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A61,0)) + SUMIFS('Credit Card 2'!D:D,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A61,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A61,0))</f>
+        <v/>
+      </c>
+      <c r="K61" s="15">
+        <f>SUMIFS('Credit Card 1'!E:E,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A61,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A61,0)) + SUMIFS('Credit Card 2'!E:E,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A61,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A61,0))</f>
+        <v/>
+      </c>
+      <c r="L61" s="15">
+        <f>SUMIFS('Credit Card 1'!F:F,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A61,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A61,0)) + SUMIFS('Credit Card 2'!F:F,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A61,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A61,0))</f>
+        <v/>
+      </c>
+      <c r="M61" s="15">
+        <f>K61+L61-J61</f>
+        <v/>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="19" t="n">
+        <v>47088</v>
+      </c>
+      <c r="B62" s="15">
+        <f>SUMIFS('Current'!D:D,'Current'!A:A,"&gt;="&amp;EOMONTH($A62,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A62,0)) + SUMIFS('Chase'!D:D,'Chase'!A:A,"&gt;="&amp;EOMONTH($A62,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A62,0)) + SUMIFS('Wellsfargo'!D:D,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A62,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A62,0)) + SUMIFS('Vyral'!D:D,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A62,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A62,0))</f>
+        <v/>
+      </c>
+      <c r="C62" s="15">
+        <f>SUMIFS('Current'!E:E,'Current'!A:A,"&gt;="&amp;EOMONTH($A62,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A62,0)) + SUMIFS('Chase'!E:E,'Chase'!A:A,"&gt;="&amp;EOMONTH($A62,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A62,0)) + SUMIFS('Wellsfargo'!E:E,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A62,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A62,0)) + SUMIFS('Vyral'!E:E,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A62,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A62,0))</f>
+        <v/>
+      </c>
+      <c r="D62" s="15">
+        <f>SUMIFS('Current'!F:F,'Current'!A:A,"&gt;="&amp;EOMONTH($A62,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A62,0)) + SUMIFS('Chase'!F:F,'Chase'!A:A,"&gt;="&amp;EOMONTH($A62,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A62,0)) + SUMIFS('Wellsfargo'!F:F,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A62,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A62,0)) + SUMIFS('Vyral'!F:F,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A62,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A62,0))</f>
+        <v/>
+      </c>
+      <c r="E62" s="15">
+        <f>B62-C62-D62</f>
+        <v/>
+      </c>
+      <c r="F62" s="9">
+        <f>SUMIFS('Ghana City'!D:D,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A62,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A62,0))</f>
+        <v/>
+      </c>
+      <c r="G62" s="9">
+        <f>SUMIFS('Ghana City'!E:E,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A62,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A62,0))</f>
+        <v/>
+      </c>
+      <c r="H62" s="9">
+        <f>SUMIFS('Ghana City'!F:F,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A62,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A62,0))</f>
+        <v/>
+      </c>
+      <c r="I62" s="9">
+        <f>F62-G62-H62</f>
+        <v/>
+      </c>
+      <c r="J62" s="15">
+        <f>SUMIFS('Credit Card 1'!D:D,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A62,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A62,0)) + SUMIFS('Credit Card 2'!D:D,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A62,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A62,0))</f>
+        <v/>
+      </c>
+      <c r="K62" s="15">
+        <f>SUMIFS('Credit Card 1'!E:E,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A62,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A62,0)) + SUMIFS('Credit Card 2'!E:E,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A62,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A62,0))</f>
+        <v/>
+      </c>
+      <c r="L62" s="15">
+        <f>SUMIFS('Credit Card 1'!F:F,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A62,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A62,0)) + SUMIFS('Credit Card 2'!F:F,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A62,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A62,0))</f>
+        <v/>
+      </c>
+      <c r="M62" s="15">
+        <f>K62+L62-J62</f>
+        <v/>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="19" t="n">
+        <v>47119</v>
+      </c>
+      <c r="B63" s="15">
+        <f>SUMIFS('Current'!D:D,'Current'!A:A,"&gt;="&amp;EOMONTH($A63,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A63,0)) + SUMIFS('Chase'!D:D,'Chase'!A:A,"&gt;="&amp;EOMONTH($A63,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A63,0)) + SUMIFS('Wellsfargo'!D:D,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A63,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A63,0)) + SUMIFS('Vyral'!D:D,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A63,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A63,0))</f>
+        <v/>
+      </c>
+      <c r="C63" s="15">
+        <f>SUMIFS('Current'!E:E,'Current'!A:A,"&gt;="&amp;EOMONTH($A63,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A63,0)) + SUMIFS('Chase'!E:E,'Chase'!A:A,"&gt;="&amp;EOMONTH($A63,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A63,0)) + SUMIFS('Wellsfargo'!E:E,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A63,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A63,0)) + SUMIFS('Vyral'!E:E,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A63,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A63,0))</f>
+        <v/>
+      </c>
+      <c r="D63" s="15">
+        <f>SUMIFS('Current'!F:F,'Current'!A:A,"&gt;="&amp;EOMONTH($A63,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A63,0)) + SUMIFS('Chase'!F:F,'Chase'!A:A,"&gt;="&amp;EOMONTH($A63,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A63,0)) + SUMIFS('Wellsfargo'!F:F,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A63,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A63,0)) + SUMIFS('Vyral'!F:F,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A63,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A63,0))</f>
+        <v/>
+      </c>
+      <c r="E63" s="15">
+        <f>B63-C63-D63</f>
+        <v/>
+      </c>
+      <c r="F63" s="9">
+        <f>SUMIFS('Ghana City'!D:D,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A63,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A63,0))</f>
+        <v/>
+      </c>
+      <c r="G63" s="9">
+        <f>SUMIFS('Ghana City'!E:E,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A63,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A63,0))</f>
+        <v/>
+      </c>
+      <c r="H63" s="9">
+        <f>SUMIFS('Ghana City'!F:F,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A63,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A63,0))</f>
+        <v/>
+      </c>
+      <c r="I63" s="9">
+        <f>F63-G63-H63</f>
+        <v/>
+      </c>
+      <c r="J63" s="15">
+        <f>SUMIFS('Credit Card 1'!D:D,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A63,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A63,0)) + SUMIFS('Credit Card 2'!D:D,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A63,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A63,0))</f>
+        <v/>
+      </c>
+      <c r="K63" s="15">
+        <f>SUMIFS('Credit Card 1'!E:E,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A63,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A63,0)) + SUMIFS('Credit Card 2'!E:E,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A63,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A63,0))</f>
+        <v/>
+      </c>
+      <c r="L63" s="15">
+        <f>SUMIFS('Credit Card 1'!F:F,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A63,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A63,0)) + SUMIFS('Credit Card 2'!F:F,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A63,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A63,0))</f>
+        <v/>
+      </c>
+      <c r="M63" s="15">
+        <f>K63+L63-J63</f>
+        <v/>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="19" t="n">
+        <v>47150</v>
+      </c>
+      <c r="B64" s="15">
+        <f>SUMIFS('Current'!D:D,'Current'!A:A,"&gt;="&amp;EOMONTH($A64,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A64,0)) + SUMIFS('Chase'!D:D,'Chase'!A:A,"&gt;="&amp;EOMONTH($A64,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A64,0)) + SUMIFS('Wellsfargo'!D:D,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A64,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A64,0)) + SUMIFS('Vyral'!D:D,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A64,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A64,0))</f>
+        <v/>
+      </c>
+      <c r="C64" s="15">
+        <f>SUMIFS('Current'!E:E,'Current'!A:A,"&gt;="&amp;EOMONTH($A64,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A64,0)) + SUMIFS('Chase'!E:E,'Chase'!A:A,"&gt;="&amp;EOMONTH($A64,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A64,0)) + SUMIFS('Wellsfargo'!E:E,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A64,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A64,0)) + SUMIFS('Vyral'!E:E,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A64,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A64,0))</f>
+        <v/>
+      </c>
+      <c r="D64" s="15">
+        <f>SUMIFS('Current'!F:F,'Current'!A:A,"&gt;="&amp;EOMONTH($A64,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A64,0)) + SUMIFS('Chase'!F:F,'Chase'!A:A,"&gt;="&amp;EOMONTH($A64,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A64,0)) + SUMIFS('Wellsfargo'!F:F,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A64,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A64,0)) + SUMIFS('Vyral'!F:F,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A64,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A64,0))</f>
+        <v/>
+      </c>
+      <c r="E64" s="15">
+        <f>B64-C64-D64</f>
+        <v/>
+      </c>
+      <c r="F64" s="9">
+        <f>SUMIFS('Ghana City'!D:D,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A64,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A64,0))</f>
+        <v/>
+      </c>
+      <c r="G64" s="9">
+        <f>SUMIFS('Ghana City'!E:E,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A64,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A64,0))</f>
+        <v/>
+      </c>
+      <c r="H64" s="9">
+        <f>SUMIFS('Ghana City'!F:F,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A64,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A64,0))</f>
+        <v/>
+      </c>
+      <c r="I64" s="9">
+        <f>F64-G64-H64</f>
+        <v/>
+      </c>
+      <c r="J64" s="15">
+        <f>SUMIFS('Credit Card 1'!D:D,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A64,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A64,0)) + SUMIFS('Credit Card 2'!D:D,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A64,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A64,0))</f>
+        <v/>
+      </c>
+      <c r="K64" s="15">
+        <f>SUMIFS('Credit Card 1'!E:E,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A64,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A64,0)) + SUMIFS('Credit Card 2'!E:E,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A64,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A64,0))</f>
+        <v/>
+      </c>
+      <c r="L64" s="15">
+        <f>SUMIFS('Credit Card 1'!F:F,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A64,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A64,0)) + SUMIFS('Credit Card 2'!F:F,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A64,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A64,0))</f>
+        <v/>
+      </c>
+      <c r="M64" s="15">
+        <f>K64+L64-J64</f>
+        <v/>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="19" t="n">
+        <v>47178</v>
+      </c>
+      <c r="B65" s="15">
+        <f>SUMIFS('Current'!D:D,'Current'!A:A,"&gt;="&amp;EOMONTH($A65,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A65,0)) + SUMIFS('Chase'!D:D,'Chase'!A:A,"&gt;="&amp;EOMONTH($A65,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A65,0)) + SUMIFS('Wellsfargo'!D:D,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A65,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A65,0)) + SUMIFS('Vyral'!D:D,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A65,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A65,0))</f>
+        <v/>
+      </c>
+      <c r="C65" s="15">
+        <f>SUMIFS('Current'!E:E,'Current'!A:A,"&gt;="&amp;EOMONTH($A65,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A65,0)) + SUMIFS('Chase'!E:E,'Chase'!A:A,"&gt;="&amp;EOMONTH($A65,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A65,0)) + SUMIFS('Wellsfargo'!E:E,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A65,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A65,0)) + SUMIFS('Vyral'!E:E,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A65,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A65,0))</f>
+        <v/>
+      </c>
+      <c r="D65" s="15">
+        <f>SUMIFS('Current'!F:F,'Current'!A:A,"&gt;="&amp;EOMONTH($A65,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A65,0)) + SUMIFS('Chase'!F:F,'Chase'!A:A,"&gt;="&amp;EOMONTH($A65,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A65,0)) + SUMIFS('Wellsfargo'!F:F,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A65,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A65,0)) + SUMIFS('Vyral'!F:F,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A65,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A65,0))</f>
+        <v/>
+      </c>
+      <c r="E65" s="15">
+        <f>B65-C65-D65</f>
+        <v/>
+      </c>
+      <c r="F65" s="9">
+        <f>SUMIFS('Ghana City'!D:D,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A65,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A65,0))</f>
+        <v/>
+      </c>
+      <c r="G65" s="9">
+        <f>SUMIFS('Ghana City'!E:E,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A65,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A65,0))</f>
+        <v/>
+      </c>
+      <c r="H65" s="9">
+        <f>SUMIFS('Ghana City'!F:F,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A65,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A65,0))</f>
+        <v/>
+      </c>
+      <c r="I65" s="9">
+        <f>F65-G65-H65</f>
+        <v/>
+      </c>
+      <c r="J65" s="15">
+        <f>SUMIFS('Credit Card 1'!D:D,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A65,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A65,0)) + SUMIFS('Credit Card 2'!D:D,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A65,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A65,0))</f>
+        <v/>
+      </c>
+      <c r="K65" s="15">
+        <f>SUMIFS('Credit Card 1'!E:E,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A65,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A65,0)) + SUMIFS('Credit Card 2'!E:E,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A65,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A65,0))</f>
+        <v/>
+      </c>
+      <c r="L65" s="15">
+        <f>SUMIFS('Credit Card 1'!F:F,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A65,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A65,0)) + SUMIFS('Credit Card 2'!F:F,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A65,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A65,0))</f>
+        <v/>
+      </c>
+      <c r="M65" s="15">
+        <f>K65+L65-J65</f>
+        <v/>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="19" t="n">
+        <v>47209</v>
+      </c>
+      <c r="B66" s="15">
+        <f>SUMIFS('Current'!D:D,'Current'!A:A,"&gt;="&amp;EOMONTH($A66,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A66,0)) + SUMIFS('Chase'!D:D,'Chase'!A:A,"&gt;="&amp;EOMONTH($A66,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A66,0)) + SUMIFS('Wellsfargo'!D:D,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A66,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A66,0)) + SUMIFS('Vyral'!D:D,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A66,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A66,0))</f>
+        <v/>
+      </c>
+      <c r="C66" s="15">
+        <f>SUMIFS('Current'!E:E,'Current'!A:A,"&gt;="&amp;EOMONTH($A66,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A66,0)) + SUMIFS('Chase'!E:E,'Chase'!A:A,"&gt;="&amp;EOMONTH($A66,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A66,0)) + SUMIFS('Wellsfargo'!E:E,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A66,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A66,0)) + SUMIFS('Vyral'!E:E,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A66,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A66,0))</f>
+        <v/>
+      </c>
+      <c r="D66" s="15">
+        <f>SUMIFS('Current'!F:F,'Current'!A:A,"&gt;="&amp;EOMONTH($A66,-1)+1,'Current'!A:A,"&lt;="&amp;EOMONTH($A66,0)) + SUMIFS('Chase'!F:F,'Chase'!A:A,"&gt;="&amp;EOMONTH($A66,-1)+1,'Chase'!A:A,"&lt;="&amp;EOMONTH($A66,0)) + SUMIFS('Wellsfargo'!F:F,'Wellsfargo'!A:A,"&gt;="&amp;EOMONTH($A66,-1)+1,'Wellsfargo'!A:A,"&lt;="&amp;EOMONTH($A66,0)) + SUMIFS('Vyral'!F:F,'Vyral'!A:A,"&gt;="&amp;EOMONTH($A66,-1)+1,'Vyral'!A:A,"&lt;="&amp;EOMONTH($A66,0))</f>
+        <v/>
+      </c>
+      <c r="E66" s="15">
+        <f>B66-C66-D66</f>
+        <v/>
+      </c>
+      <c r="F66" s="9">
+        <f>SUMIFS('Ghana City'!D:D,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A66,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A66,0))</f>
+        <v/>
+      </c>
+      <c r="G66" s="9">
+        <f>SUMIFS('Ghana City'!E:E,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A66,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A66,0))</f>
+        <v/>
+      </c>
+      <c r="H66" s="9">
+        <f>SUMIFS('Ghana City'!F:F,'Ghana City'!A:A,"&gt;="&amp;EOMONTH($A66,-1)+1,'Ghana City'!A:A,"&lt;="&amp;EOMONTH($A66,0))</f>
+        <v/>
+      </c>
+      <c r="I66" s="9">
+        <f>F66-G66-H66</f>
+        <v/>
+      </c>
+      <c r="J66" s="15">
+        <f>SUMIFS('Credit Card 1'!D:D,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A66,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A66,0)) + SUMIFS('Credit Card 2'!D:D,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A66,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A66,0))</f>
+        <v/>
+      </c>
+      <c r="K66" s="15">
+        <f>SUMIFS('Credit Card 1'!E:E,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A66,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A66,0)) + SUMIFS('Credit Card 2'!E:E,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A66,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A66,0))</f>
+        <v/>
+      </c>
+      <c r="L66" s="15">
+        <f>SUMIFS('Credit Card 1'!F:F,'Credit Card 1'!A:A,"&gt;="&amp;EOMONTH($A66,-1)+1,'Credit Card 1'!A:A,"&lt;="&amp;EOMONTH($A66,0)) + SUMIFS('Credit Card 2'!F:F,'Credit Card 2'!A:A,"&gt;="&amp;EOMONTH($A66,-1)+1,'Credit Card 2'!A:A,"&lt;="&amp;EOMONTH($A66,0))</f>
+        <v/>
+      </c>
+      <c r="M66" s="15">
+        <f>K66+L66-J66</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Collapse timeline section by default on summary dashboard
Co-authored-by: Samuel Kafui Kwawukume <samkafs@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/personal_finance_tracker.xlsx
+++ b/personal_finance_tracker.xlsx
@@ -509,6 +509,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -692,6 +693,7 @@
         <v/>
       </c>
     </row>
+    <row r="12"/>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
@@ -715,6 +717,8 @@
         <v/>
       </c>
     </row>
+    <row r="14"/>
+    <row r="15"/>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
@@ -772,6 +776,8 @@
         <v/>
       </c>
     </row>
+    <row r="19"/>
+    <row r="20"/>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
@@ -852,14 +858,22 @@
         <v/>
       </c>
     </row>
+    <row r="25"/>
+    <row r="26"/>
+    <row r="27"/>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>Monthly Timeline (Apr 2026 to Apr 2029)</t>
+          <t>Monthly Timeline (Apr 2026 to Apr 2029) - collapsed by default</t>
         </is>
       </c>
-    </row>
-    <row r="29">
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>Click + on left margin to expand timeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" hidden="1" outlineLevel="1">
       <c r="A29" s="5" t="inlineStr">
         <is>
           <t>Month</t>
@@ -926,7 +940,7 @@
         </is>
       </c>
     </row>
-    <row r="30">
+    <row r="30" hidden="1" outlineLevel="1">
       <c r="A30" s="19" t="n">
         <v>46113</v>
       </c>
@@ -979,7 +993,7 @@
         <v/>
       </c>
     </row>
-    <row r="31">
+    <row r="31" hidden="1" outlineLevel="1">
       <c r="A31" s="19" t="n">
         <v>46143</v>
       </c>
@@ -1032,7 +1046,7 @@
         <v/>
       </c>
     </row>
-    <row r="32">
+    <row r="32" hidden="1" outlineLevel="1">
       <c r="A32" s="19" t="n">
         <v>46174</v>
       </c>
@@ -1085,7 +1099,7 @@
         <v/>
       </c>
     </row>
-    <row r="33">
+    <row r="33" hidden="1" outlineLevel="1">
       <c r="A33" s="19" t="n">
         <v>46204</v>
       </c>
@@ -1138,7 +1152,7 @@
         <v/>
       </c>
     </row>
-    <row r="34">
+    <row r="34" hidden="1" outlineLevel="1">
       <c r="A34" s="19" t="n">
         <v>46235</v>
       </c>
@@ -1191,7 +1205,7 @@
         <v/>
       </c>
     </row>
-    <row r="35">
+    <row r="35" hidden="1" outlineLevel="1">
       <c r="A35" s="19" t="n">
         <v>46266</v>
       </c>
@@ -1244,7 +1258,7 @@
         <v/>
       </c>
     </row>
-    <row r="36">
+    <row r="36" hidden="1" outlineLevel="1">
       <c r="A36" s="19" t="n">
         <v>46296</v>
       </c>
@@ -1297,7 +1311,7 @@
         <v/>
       </c>
     </row>
-    <row r="37">
+    <row r="37" hidden="1" outlineLevel="1">
       <c r="A37" s="19" t="n">
         <v>46327</v>
       </c>
@@ -1350,7 +1364,7 @@
         <v/>
       </c>
     </row>
-    <row r="38">
+    <row r="38" hidden="1" outlineLevel="1">
       <c r="A38" s="19" t="n">
         <v>46357</v>
       </c>
@@ -1403,7 +1417,7 @@
         <v/>
       </c>
     </row>
-    <row r="39">
+    <row r="39" hidden="1" outlineLevel="1">
       <c r="A39" s="19" t="n">
         <v>46388</v>
       </c>
@@ -1456,7 +1470,7 @@
         <v/>
       </c>
     </row>
-    <row r="40">
+    <row r="40" hidden="1" outlineLevel="1">
       <c r="A40" s="19" t="n">
         <v>46419</v>
       </c>
@@ -1509,7 +1523,7 @@
         <v/>
       </c>
     </row>
-    <row r="41">
+    <row r="41" hidden="1" outlineLevel="1">
       <c r="A41" s="19" t="n">
         <v>46447</v>
       </c>
@@ -1562,7 +1576,7 @@
         <v/>
       </c>
     </row>
-    <row r="42">
+    <row r="42" hidden="1" outlineLevel="1">
       <c r="A42" s="19" t="n">
         <v>46478</v>
       </c>
@@ -1615,7 +1629,7 @@
         <v/>
       </c>
     </row>
-    <row r="43">
+    <row r="43" hidden="1" outlineLevel="1">
       <c r="A43" s="19" t="n">
         <v>46508</v>
       </c>
@@ -1668,7 +1682,7 @@
         <v/>
       </c>
     </row>
-    <row r="44">
+    <row r="44" hidden="1" outlineLevel="1">
       <c r="A44" s="19" t="n">
         <v>46539</v>
       </c>
@@ -1721,7 +1735,7 @@
         <v/>
       </c>
     </row>
-    <row r="45">
+    <row r="45" hidden="1" outlineLevel="1">
       <c r="A45" s="19" t="n">
         <v>46569</v>
       </c>
@@ -1774,7 +1788,7 @@
         <v/>
       </c>
     </row>
-    <row r="46">
+    <row r="46" hidden="1" outlineLevel="1">
       <c r="A46" s="19" t="n">
         <v>46600</v>
       </c>
@@ -1827,7 +1841,7 @@
         <v/>
       </c>
     </row>
-    <row r="47">
+    <row r="47" hidden="1" outlineLevel="1">
       <c r="A47" s="19" t="n">
         <v>46631</v>
       </c>
@@ -1880,7 +1894,7 @@
         <v/>
       </c>
     </row>
-    <row r="48">
+    <row r="48" hidden="1" outlineLevel="1">
       <c r="A48" s="19" t="n">
         <v>46661</v>
       </c>
@@ -1933,7 +1947,7 @@
         <v/>
       </c>
     </row>
-    <row r="49">
+    <row r="49" hidden="1" outlineLevel="1">
       <c r="A49" s="19" t="n">
         <v>46692</v>
       </c>
@@ -1986,7 +2000,7 @@
         <v/>
       </c>
     </row>
-    <row r="50">
+    <row r="50" hidden="1" outlineLevel="1">
       <c r="A50" s="19" t="n">
         <v>46722</v>
       </c>
@@ -2039,7 +2053,7 @@
         <v/>
       </c>
     </row>
-    <row r="51">
+    <row r="51" hidden="1" outlineLevel="1">
       <c r="A51" s="19" t="n">
         <v>46753</v>
       </c>
@@ -2092,7 +2106,7 @@
         <v/>
       </c>
     </row>
-    <row r="52">
+    <row r="52" hidden="1" outlineLevel="1">
       <c r="A52" s="19" t="n">
         <v>46784</v>
       </c>
@@ -2145,7 +2159,7 @@
         <v/>
       </c>
     </row>
-    <row r="53">
+    <row r="53" hidden="1" outlineLevel="1">
       <c r="A53" s="19" t="n">
         <v>46813</v>
       </c>
@@ -2198,7 +2212,7 @@
         <v/>
       </c>
     </row>
-    <row r="54">
+    <row r="54" hidden="1" outlineLevel="1">
       <c r="A54" s="19" t="n">
         <v>46844</v>
       </c>
@@ -2251,7 +2265,7 @@
         <v/>
       </c>
     </row>
-    <row r="55">
+    <row r="55" hidden="1" outlineLevel="1">
       <c r="A55" s="19" t="n">
         <v>46874</v>
       </c>
@@ -2304,7 +2318,7 @@
         <v/>
       </c>
     </row>
-    <row r="56">
+    <row r="56" hidden="1" outlineLevel="1">
       <c r="A56" s="19" t="n">
         <v>46905</v>
       </c>
@@ -2357,7 +2371,7 @@
         <v/>
       </c>
     </row>
-    <row r="57">
+    <row r="57" hidden="1" outlineLevel="1">
       <c r="A57" s="19" t="n">
         <v>46935</v>
       </c>
@@ -2410,7 +2424,7 @@
         <v/>
       </c>
     </row>
-    <row r="58">
+    <row r="58" hidden="1" outlineLevel="1">
       <c r="A58" s="19" t="n">
         <v>46966</v>
       </c>
@@ -2463,7 +2477,7 @@
         <v/>
       </c>
     </row>
-    <row r="59">
+    <row r="59" hidden="1" outlineLevel="1">
       <c r="A59" s="19" t="n">
         <v>46997</v>
       </c>
@@ -2516,7 +2530,7 @@
         <v/>
       </c>
     </row>
-    <row r="60">
+    <row r="60" hidden="1" outlineLevel="1">
       <c r="A60" s="19" t="n">
         <v>47027</v>
       </c>
@@ -2569,7 +2583,7 @@
         <v/>
       </c>
     </row>
-    <row r="61">
+    <row r="61" hidden="1" outlineLevel="1">
       <c r="A61" s="19" t="n">
         <v>47058</v>
       </c>
@@ -2622,7 +2636,7 @@
         <v/>
       </c>
     </row>
-    <row r="62">
+    <row r="62" hidden="1" outlineLevel="1">
       <c r="A62" s="19" t="n">
         <v>47088</v>
       </c>
@@ -2675,7 +2689,7 @@
         <v/>
       </c>
     </row>
-    <row r="63">
+    <row r="63" hidden="1" outlineLevel="1">
       <c r="A63" s="19" t="n">
         <v>47119</v>
       </c>
@@ -2728,7 +2742,7 @@
         <v/>
       </c>
     </row>
-    <row r="64">
+    <row r="64" hidden="1" outlineLevel="1">
       <c r="A64" s="19" t="n">
         <v>47150</v>
       </c>
@@ -2781,7 +2795,7 @@
         <v/>
       </c>
     </row>
-    <row r="65">
+    <row r="65" hidden="1" outlineLevel="1">
       <c r="A65" s="19" t="n">
         <v>47178</v>
       </c>
@@ -2834,7 +2848,7 @@
         <v/>
       </c>
     </row>
-    <row r="66">
+    <row r="66" hidden="1" outlineLevel="1">
       <c r="A66" s="19" t="n">
         <v>47209</v>
       </c>

</xml_diff>

<commit_message>
Restore current balance snapshot section on summary dashboard
Co-authored-by: Samuel Kafui Kwawukume <samkafs@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/personal_finance_tracker.xlsx
+++ b/personal_finance_tracker.xlsx
@@ -96,7 +96,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -119,6 +119,8 @@
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -493,10 +495,10 @@
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="28" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="38" customWidth="1" min="10" max="10"/>
     <col width="14" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
     <col width="20" customWidth="1" min="13" max="13"/>
@@ -505,11 +507,10 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Monthly Flow Dashboard (Month-Only)</t>
+          <t>Finance Dashboard (Monthly Flow + Current Balances)</t>
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -519,9 +520,14 @@
       <c r="C3" s="14" t="n">
         <v>46113</v>
       </c>
+      <c r="G3" s="4" t="inlineStr">
+        <is>
+          <t>Current Balance Snapshot</t>
+        </is>
+      </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>How it works</t>
+          <t>How to use</t>
         </is>
       </c>
     </row>
@@ -544,16 +550,45 @@
         <f>EOMONTH(C3,0)</f>
         <v/>
       </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>Account</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>Current Balance / Owed</t>
+        </is>
+      </c>
+      <c r="I4" s="5" t="inlineStr">
+        <is>
+          <t>Currency</t>
+        </is>
+      </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>1) Change C3 to any date in a month</t>
+          <t>1) C3 selects month for monthly tables</t>
         </is>
       </c>
     </row>
     <row r="5">
+      <c r="G5" s="6" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="H5" s="15">
+        <f>'Current'!B4</f>
+        <v/>
+      </c>
+      <c r="I5" s="6" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2) Selected-month tables update automatically</t>
+          <t>2) Left tables = selected month flows only</t>
         </is>
       </c>
     </row>
@@ -563,9 +598,23 @@
           <t>Selected Month - USD Bank Accounts</t>
         </is>
       </c>
+      <c r="G6" s="6" t="inlineStr">
+        <is>
+          <t>Chase</t>
+        </is>
+      </c>
+      <c r="H6" s="15">
+        <f>'Chase'!B4</f>
+        <v/>
+      </c>
+      <c r="I6" s="6" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>3) Timeline is auto-filled Apr 2026-Apr 2029</t>
+          <t>3) Right panel = current balances snapshot</t>
         </is>
       </c>
     </row>
@@ -595,9 +644,23 @@
           <t>Net Flow</t>
         </is>
       </c>
+      <c r="G7" s="6" t="inlineStr">
+        <is>
+          <t>Wellsfargo</t>
+        </is>
+      </c>
+      <c r="H7" s="15">
+        <f>'Wellsfargo'!B4</f>
+        <v/>
+      </c>
+      <c r="I7" s="6" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>4) No current balance columns are shown</t>
+          <t>4) Timeline is collapsed (use + to expand)</t>
         </is>
       </c>
     </row>
@@ -623,6 +686,20 @@
         <f>B8-C8-D8</f>
         <v/>
       </c>
+      <c r="G8" s="6" t="inlineStr">
+        <is>
+          <t>Vyral</t>
+        </is>
+      </c>
+      <c r="H8" s="15">
+        <f>'Vyral'!B4</f>
+        <v/>
+      </c>
+      <c r="I8" s="6" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
@@ -646,6 +723,20 @@
         <f>B9-C9-D9</f>
         <v/>
       </c>
+      <c r="G9" s="20" t="inlineStr">
+        <is>
+          <t>Total USD Bank Balance</t>
+        </is>
+      </c>
+      <c r="H9" s="21">
+        <f>SUM(H5:H8)</f>
+        <v/>
+      </c>
+      <c r="I9" s="20" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
@@ -692,8 +783,21 @@
         <f>B11-C11-D11</f>
         <v/>
       </c>
-    </row>
-    <row r="12"/>
+      <c r="G11" s="6" t="inlineStr">
+        <is>
+          <t>Ghana City (Bank)</t>
+        </is>
+      </c>
+      <c r="H11" s="9">
+        <f>'Ghana City'!B4</f>
+        <v/>
+      </c>
+      <c r="I11" s="6" t="inlineStr">
+        <is>
+          <t>GHS</t>
+        </is>
+      </c>
+    </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
@@ -716,15 +820,73 @@
         <f>SUM(E8:E11)</f>
         <v/>
       </c>
-    </row>
-    <row r="14"/>
-    <row r="15"/>
+      <c r="G13" s="6" t="inlineStr">
+        <is>
+          <t>Credit Card 1 (Owed)</t>
+        </is>
+      </c>
+      <c r="H13" s="15">
+        <f>'Credit Card 1'!B4</f>
+        <v/>
+      </c>
+      <c r="I13" s="6" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="G14" s="6" t="inlineStr">
+        <is>
+          <t>Credit Card 2 (Owed)</t>
+        </is>
+      </c>
+      <c r="H14" s="15">
+        <f>'Credit Card 2'!B4</f>
+        <v/>
+      </c>
+      <c r="I14" s="6" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="G15" s="20" t="inlineStr">
+        <is>
+          <t>Total Credit Cards Owed</t>
+        </is>
+      </c>
+      <c r="H15" s="21">
+        <f>H13+H14</f>
+        <v/>
+      </c>
+      <c r="I15" s="20" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+    </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
           <t>Selected Month - GHS Bank Accounts</t>
         </is>
       </c>
+      <c r="G16" s="20" t="inlineStr">
+        <is>
+          <t>Net USD Position (Banks - Cards)</t>
+        </is>
+      </c>
+      <c r="H16" s="21">
+        <f>H9-H15</f>
+        <v/>
+      </c>
+      <c r="I16" s="20" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
@@ -776,8 +938,6 @@
         <v/>
       </c>
     </row>
-    <row r="19"/>
-    <row r="20"/>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
@@ -858,9 +1018,6 @@
         <v/>
       </c>
     </row>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Add monthly start balance columns to selected-month summary tables
Co-authored-by: Samuel Kafui Kwawukume <samkafs@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/personal_finance_tracker.xlsx
+++ b/personal_finance_tracker.xlsx
@@ -491,10 +491,10 @@
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
     <col width="28" customWidth="1" min="7" max="7"/>
     <col width="24" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
@@ -626,20 +626,25 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
+          <t>Start Balance</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
           <t>Money In</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr">
+      <c r="D7" s="5" t="inlineStr">
         <is>
           <t>Money Out</t>
         </is>
       </c>
-      <c r="D7" s="5" t="inlineStr">
+      <c r="E7" s="5" t="inlineStr">
         <is>
           <t>Tax</t>
         </is>
       </c>
-      <c r="E7" s="5" t="inlineStr">
+      <c r="F7" s="5" t="inlineStr">
         <is>
           <t>Net Flow</t>
         </is>
@@ -671,19 +676,23 @@
         </is>
       </c>
       <c r="B8" s="15">
+        <f>IFERROR(LOOKUP(2,1/(('Current'!A:A&lt;$B$4)*('Current'!G:G&lt;&gt;"")),'Current'!G:G),'Current'!B3)</f>
+        <v/>
+      </c>
+      <c r="C8" s="15">
         <f>SUMIFS('Current'!D:D,'Current'!A:A,"&gt;="&amp;$B$4,'Current'!A:A,"&lt;="&amp;$D$4)</f>
         <v/>
       </c>
-      <c r="C8" s="15">
+      <c r="D8" s="15">
         <f>SUMIFS('Current'!E:E,'Current'!A:A,"&gt;="&amp;$B$4,'Current'!A:A,"&lt;="&amp;$D$4)</f>
         <v/>
       </c>
-      <c r="D8" s="15">
+      <c r="E8" s="15">
         <f>SUMIFS('Current'!F:F,'Current'!A:A,"&gt;="&amp;$B$4,'Current'!A:A,"&lt;="&amp;$D$4)</f>
         <v/>
       </c>
-      <c r="E8" s="15">
-        <f>B8-C8-D8</f>
+      <c r="F8" s="15">
+        <f>C8-D8-E8</f>
         <v/>
       </c>
       <c r="G8" s="6" t="inlineStr">
@@ -708,19 +717,23 @@
         </is>
       </c>
       <c r="B9" s="15">
+        <f>IFERROR(LOOKUP(2,1/(('Chase'!A:A&lt;$B$4)*('Chase'!G:G&lt;&gt;"")),'Chase'!G:G),'Chase'!B3)</f>
+        <v/>
+      </c>
+      <c r="C9" s="15">
         <f>SUMIFS('Chase'!D:D,'Chase'!A:A,"&gt;="&amp;$B$4,'Chase'!A:A,"&lt;="&amp;$D$4)</f>
         <v/>
       </c>
-      <c r="C9" s="15">
+      <c r="D9" s="15">
         <f>SUMIFS('Chase'!E:E,'Chase'!A:A,"&gt;="&amp;$B$4,'Chase'!A:A,"&lt;="&amp;$D$4)</f>
         <v/>
       </c>
-      <c r="D9" s="15">
+      <c r="E9" s="15">
         <f>SUMIFS('Chase'!F:F,'Chase'!A:A,"&gt;="&amp;$B$4,'Chase'!A:A,"&lt;="&amp;$D$4)</f>
         <v/>
       </c>
-      <c r="E9" s="15">
-        <f>B9-C9-D9</f>
+      <c r="F9" s="15">
+        <f>C9-D9-E9</f>
         <v/>
       </c>
       <c r="G9" s="20" t="inlineStr">
@@ -745,19 +758,23 @@
         </is>
       </c>
       <c r="B10" s="15">
+        <f>IFERROR(LOOKUP(2,1/(('Wellsfargo'!A:A&lt;$B$4)*('Wellsfargo'!G:G&lt;&gt;"")),'Wellsfargo'!G:G),'Wellsfargo'!B3)</f>
+        <v/>
+      </c>
+      <c r="C10" s="15">
         <f>SUMIFS('Wellsfargo'!D:D,'Wellsfargo'!A:A,"&gt;="&amp;$B$4,'Wellsfargo'!A:A,"&lt;="&amp;$D$4)</f>
         <v/>
       </c>
-      <c r="C10" s="15">
+      <c r="D10" s="15">
         <f>SUMIFS('Wellsfargo'!E:E,'Wellsfargo'!A:A,"&gt;="&amp;$B$4,'Wellsfargo'!A:A,"&lt;="&amp;$D$4)</f>
         <v/>
       </c>
-      <c r="D10" s="15">
+      <c r="E10" s="15">
         <f>SUMIFS('Wellsfargo'!F:F,'Wellsfargo'!A:A,"&gt;="&amp;$B$4,'Wellsfargo'!A:A,"&lt;="&amp;$D$4)</f>
         <v/>
       </c>
-      <c r="E10" s="15">
-        <f>B10-C10-D10</f>
+      <c r="F10" s="15">
+        <f>C10-D10-E10</f>
         <v/>
       </c>
     </row>
@@ -768,19 +785,23 @@
         </is>
       </c>
       <c r="B11" s="15">
+        <f>IFERROR(LOOKUP(2,1/(('Vyral'!A:A&lt;$B$4)*('Vyral'!G:G&lt;&gt;"")),'Vyral'!G:G),'Vyral'!B3)</f>
+        <v/>
+      </c>
+      <c r="C11" s="15">
         <f>SUMIFS('Vyral'!D:D,'Vyral'!A:A,"&gt;="&amp;$B$4,'Vyral'!A:A,"&lt;="&amp;$D$4)</f>
         <v/>
       </c>
-      <c r="C11" s="15">
+      <c r="D11" s="15">
         <f>SUMIFS('Vyral'!E:E,'Vyral'!A:A,"&gt;="&amp;$B$4,'Vyral'!A:A,"&lt;="&amp;$D$4)</f>
         <v/>
       </c>
-      <c r="D11" s="15">
+      <c r="E11" s="15">
         <f>SUMIFS('Vyral'!F:F,'Vyral'!A:A,"&gt;="&amp;$B$4,'Vyral'!A:A,"&lt;="&amp;$D$4)</f>
         <v/>
       </c>
-      <c r="E11" s="15">
-        <f>B11-C11-D11</f>
+      <c r="F11" s="15">
+        <f>C11-D11-E11</f>
         <v/>
       </c>
       <c r="G11" s="6" t="inlineStr">
@@ -820,6 +841,10 @@
         <f>SUM(E8:E11)</f>
         <v/>
       </c>
+      <c r="F13" s="16">
+        <f>SUM(F8:F11)</f>
+        <v/>
+      </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
           <t>Credit Card 1 (Owed)</t>
@@ -896,20 +921,25 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
+          <t>Start Balance</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
           <t>Money In</t>
         </is>
       </c>
-      <c r="C17" s="5" t="inlineStr">
+      <c r="D17" s="5" t="inlineStr">
         <is>
           <t>Money Out</t>
         </is>
       </c>
-      <c r="D17" s="5" t="inlineStr">
+      <c r="E17" s="5" t="inlineStr">
         <is>
           <t>Tax</t>
         </is>
       </c>
-      <c r="E17" s="5" t="inlineStr">
+      <c r="F17" s="5" t="inlineStr">
         <is>
           <t>Net Flow</t>
         </is>
@@ -922,19 +952,23 @@
         </is>
       </c>
       <c r="B18" s="9">
+        <f>IFERROR(LOOKUP(2,1/(('Ghana City'!A:A&lt;$B$4)*('Ghana City'!G:G&lt;&gt;"")),'Ghana City'!G:G),'Ghana City'!B3)</f>
+        <v/>
+      </c>
+      <c r="C18" s="9">
         <f>SUMIFS('Ghana City'!D:D,'Ghana City'!A:A,"&gt;="&amp;$B$4,'Ghana City'!A:A,"&lt;="&amp;$D$4)</f>
         <v/>
       </c>
-      <c r="C18" s="9">
+      <c r="D18" s="9">
         <f>SUMIFS('Ghana City'!E:E,'Ghana City'!A:A,"&gt;="&amp;$B$4,'Ghana City'!A:A,"&lt;="&amp;$D$4)</f>
         <v/>
       </c>
-      <c r="D18" s="9">
+      <c r="E18" s="9">
         <f>SUMIFS('Ghana City'!F:F,'Ghana City'!A:A,"&gt;="&amp;$B$4,'Ghana City'!A:A,"&lt;="&amp;$D$4)</f>
         <v/>
       </c>
-      <c r="E18" s="9">
-        <f>B18-C18-D18</f>
+      <c r="F18" s="9">
+        <f>C18-D18-E18</f>
         <v/>
       </c>
     </row>
@@ -953,20 +987,25 @@
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
+          <t>Start Owed</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
           <t>Payments In</t>
         </is>
       </c>
-      <c r="C22" s="5" t="inlineStr">
+      <c r="D22" s="5" t="inlineStr">
         <is>
           <t>Spend Out</t>
         </is>
       </c>
-      <c r="D22" s="5" t="inlineStr">
+      <c r="E22" s="5" t="inlineStr">
         <is>
           <t>Tax</t>
         </is>
       </c>
-      <c r="E22" s="5" t="inlineStr">
+      <c r="F22" s="5" t="inlineStr">
         <is>
           <t>Net Owed Change</t>
         </is>
@@ -979,19 +1018,23 @@
         </is>
       </c>
       <c r="B23" s="15">
+        <f>IFERROR(LOOKUP(2,1/(('Credit Card 1'!A:A&lt;$B$4)*('Credit Card 1'!G:G&lt;&gt;"")),'Credit Card 1'!G:G),'Credit Card 1'!B3)</f>
+        <v/>
+      </c>
+      <c r="C23" s="15">
         <f>SUMIFS('Credit Card 1'!D:D,'Credit Card 1'!A:A,"&gt;="&amp;$B$4,'Credit Card 1'!A:A,"&lt;="&amp;$D$4)</f>
         <v/>
       </c>
-      <c r="C23" s="15">
+      <c r="D23" s="15">
         <f>SUMIFS('Credit Card 1'!E:E,'Credit Card 1'!A:A,"&gt;="&amp;$B$4,'Credit Card 1'!A:A,"&lt;="&amp;$D$4)</f>
         <v/>
       </c>
-      <c r="D23" s="15">
+      <c r="E23" s="15">
         <f>SUMIFS('Credit Card 1'!F:F,'Credit Card 1'!A:A,"&gt;="&amp;$B$4,'Credit Card 1'!A:A,"&lt;="&amp;$D$4)</f>
         <v/>
       </c>
-      <c r="E23" s="15">
-        <f>C23+D23-B23</f>
+      <c r="F23" s="15">
+        <f>D23+E23-C23</f>
         <v/>
       </c>
     </row>
@@ -1002,19 +1045,23 @@
         </is>
       </c>
       <c r="B24" s="15">
+        <f>IFERROR(LOOKUP(2,1/(('Credit Card 2'!A:A&lt;$B$4)*('Credit Card 2'!G:G&lt;&gt;"")),'Credit Card 2'!G:G),'Credit Card 2'!B3)</f>
+        <v/>
+      </c>
+      <c r="C24" s="15">
         <f>SUMIFS('Credit Card 2'!D:D,'Credit Card 2'!A:A,"&gt;="&amp;$B$4,'Credit Card 2'!A:A,"&lt;="&amp;$D$4)</f>
         <v/>
       </c>
-      <c r="C24" s="15">
+      <c r="D24" s="15">
         <f>SUMIFS('Credit Card 2'!E:E,'Credit Card 2'!A:A,"&gt;="&amp;$B$4,'Credit Card 2'!A:A,"&lt;="&amp;$D$4)</f>
         <v/>
       </c>
-      <c r="D24" s="15">
+      <c r="E24" s="15">
         <f>SUMIFS('Credit Card 2'!F:F,'Credit Card 2'!A:A,"&gt;="&amp;$B$4,'Credit Card 2'!A:A,"&lt;="&amp;$D$4)</f>
         <v/>
       </c>
-      <c r="E24" s="15">
-        <f>C24+D24-B24</f>
+      <c r="F24" s="15">
+        <f>D24+E24-C24</f>
         <v/>
       </c>
     </row>

</xml_diff>